<commit_message>
Update gender classification: Female 93, Male 111, Total 204
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -617,11 +617,11 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1. นางสาวเพ็ญนภา บุญเสริม (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางราวี เวียงสมุทร (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายถาวร เวียงสมุทร (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-4. นางภิรมณ์พร บุญจันที (45–59 ปี, ครูผู้ช่วย)
-5. นางสาวกัญญารัตน์ อัมไพ (15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางสาวเพ็ญนภา บุญเสริม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางราวี เวียงสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายถาวร เวียงสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+4. นางภิรมณ์พร บุญจันที (หญิง, 45–59 ปี, ครูผู้ช่วย)
+5. นางสาวกัญญารัตน์ อัมไพ (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
@@ -707,9 +707,9 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>1. นฤมล บุญรอด (45–59 ปี, ไม่ได้ประกอบอาชีพ)
-2. อำนวย นามนาค (45–59 ปี, พนักงานบริษัท)
-3. สุวิลักขณ์ นามนาค (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นฤมล บุญรอด (หญิง, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
+2. อำนวย นามนาค (ชาย, 45–59 ปี, พนักงานบริษัท)
+3. สุวิลักขณ์ นามนาค (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G3" s="4" t="n">
@@ -795,10 +795,10 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1. นายทองคำ เลิศพาณุมาศ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสุมาลี พวงโคสน (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายประสิทธิ์ เลิศพาณุมาศ (25–44 ปี, ไม่ได้ประกอบอาชีพ)
-4. ด.ช.ปนชัย เลิศพาณุมาศ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นายทองคำ เลิศพาณุมาศ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางสุมาลี พวงโคสน (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายประสิทธิ์ เลิศพาณุมาศ (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)
+4. ด.ช.ปนชัย เลิศพาณุมาศ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
@@ -884,9 +884,9 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวบุษรา เพชรรัตน์ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นางทองอยู่ เพชรรัตน์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายอารมณ์ เพชรรัตน์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวบุษรา เพชรรัตน์ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นางทองอยู่ เพชรรัตน์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายอารมณ์ เพชรรัตน์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G5" s="4" t="n">
@@ -972,8 +972,8 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1. เล็ก สมบัติเปี่ยม (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. เยียน สมบัติเปี่ยม (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. เล็ก สมบัติเปี่ยม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. เยียน สมบัติเปี่ยม (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
@@ -1059,10 +1059,10 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>1. นายนุกุล อยู่สุข (60 ปีขึ้นไป, เกษตรกรรม)
-2. นางนงนุช อยู่สุข (45–59 ปี, เกษตรกรรม)
-3. นายธนดล อยู่สุข (25–44 ปี, เกษตรกรรม)
-4. นางวรัญธร อยู่สุข (25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายนุกุล อยู่สุข (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+2. นางนงนุช อยู่สุข (ชาย, 45–59 ปี, เกษตรกรรม)
+3. นายธนดล อยู่สุข (ชาย, 25–44 ปี, เกษตรกรรม)
+4. นางวรัญธร อยู่สุข (หญิง, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G7" s="4" t="n">
@@ -1148,9 +1148,9 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>1. นาง ฉลวย รัตนะ (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายอำนาจนายอำนาจ พรมทัศน์ (25–44 ปี, รับจ้าง)
-3. เด็กหญิงธิติมา สาธุจรัญ (15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นาง ฉลวย รัตนะ (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายอำนาจนายอำนาจ พรมทัศน์ (ชาย, 25–44 ปี, รับจ้าง)
+3. เด็กหญิงธิติมา สาธุจรัญ (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
@@ -1236,9 +1236,9 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>1. นางสุชิน  ชีวงค์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นายอนุชา เพชรรัตน์ (45–59 ปี, รับจ้าง)
-3. นายภควัฒน์ หนองใหญ่ (15–24 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสุชิน  ชีวงค์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นายอนุชา เพชรรัตน์ (ชาย, 45–59 ปี, รับจ้าง)
+3. นายภควัฒน์ หนองใหญ่ (ชาย, 15–24 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
@@ -1324,10 +1324,10 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>1. เพลินจิต ทองเจือ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. สมนึก ทองเจือ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. ภัควัตร ทองเจือ (25–44 ปี, รับจ้าง)
-4. สมคิด ทองเจือ (60 ปีขึ้นไป, รับจ้าง)</t>
+          <t>1. เพลินจิต ทองเจือ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. สมนึก ทองเจือ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. ภัควัตร ทองเจือ (ชาย, 25–44 ปี, รับจ้าง)
+4. สมคิด ทองเจือ (หญิง, 60 ปีขึ้นไป, รับจ้าง)</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวสุชิรา รื่นเริง (45–59 ปี, ช่วยเลี้ยงหลาน)</t>
+          <t>1. นางสาวสุชิรา รื่นเริง (หญิง, 45–59 ปี, ช่วยเลี้ยงหลาน)</t>
         </is>
       </c>
       <c r="G11" s="4" t="n">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>1. นายถวัลย์ คำประสิทธิ์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางไพรัตน์ คำประสิทธิ์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายกิตติพงศ์ คำประสิทธิ์ (45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. นายพงศธร คำประสิทธิ์ (45–59 ปี, รับจ้าง)
-5. นางกมลรัตน์ คำประสิทธิ์ (45–59 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
+          <t>1. นายถวัลย์ คำประสิทธิ์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางไพรัตน์ คำประสิทธิ์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายกิตติพงศ์ คำประสิทธิ์ (ชาย, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. นายพงศธร คำประสิทธิ์ (ชาย, 45–59 ปี, รับจ้าง)
+5. นางกมลรัตน์ คำประสิทธิ์ (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
@@ -1589,8 +1589,8 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>1. บุปผา ทิพย์กานนท์ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. เฉลิมพล ทิพย์กานนท์ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. บุปผา ทิพย์กานนท์ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. เฉลิมพล ทิพย์กานนท์ (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G13" s="4" t="n">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>1. นางสวง ช่วยรักษา (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสวง ช่วยรักษา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
@@ -1762,9 +1762,9 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>1. นางสำนางสำรวย เมตตา (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. นานปนวรรณ สาแหลกทอง (25–44 ปี, ไม่ได้ประกอบอาชีพ)
-3. นายจตุรงค์ เมตตา (25–44 ปี, รปภ.)</t>
+          <t>1. นางสำนางสำรวย เมตตา (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. นานปนวรรณ สาแหลกทอง (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายจตุรงค์ เมตตา (ชาย, 25–44 ปี, รปภ.)</t>
         </is>
       </c>
       <c r="G15" s="4" t="n">
@@ -1846,10 +1846,10 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>1. นางจุฑารัตน์ บุญคำ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายสมศักดิ์ ฉั่วยู่เน้ย (45–59 ปี, รับจ้าง)
-3. นายธนดล ฉั่วยู่เน้ย (25–44 ปี, รับจ้าง)
-4. นางสาวอินทิรา ฉั่วยู่เน้ย (15–24 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางจุฑารัตน์ บุญคำ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายสมศักดิ์ ฉั่วยู่เน้ย (ชาย, 45–59 ปี, รับจ้าง)
+3. นายธนดล ฉั่วยู่เน้ย (ชาย, 25–44 ปี, รับจ้าง)
+4. นางสาวอินทิรา ฉั่วยู่เน้ย (หญิง, 15–24 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
@@ -1935,10 +1935,10 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>1. ประเทือง พูลศิริ (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. เฉลิม พูลศิริ (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. เอมอร (45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. บรรพต ทองอินทร์ (60 ปีขึ้นไป, รับราชการ/รัฐวิสาหกิจ)</t>
+          <t>1. ประเทือง พูลศิริ (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. เฉลิม พูลศิริ (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+3. เอมอร (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. บรรพต ทองอินทร์ (ชาย, 60 ปีขึ้นไป, รับราชการ/รัฐวิสาหกิจ)</t>
         </is>
       </c>
       <c r="G17" s="4" t="n">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>1. นางอำพร คงผ่องแผ้ว (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. นางอำพร คงผ่องแผ้ว (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
@@ -2110,11 +2110,11 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>1. นางบุญเรือง พรมทัศน์ (60 ปีขึ้นไป, รับจ้าง)
-2. นางสาวมยุรีย์ พรมทัศน์ (60 ปีขึ้นไป, รับจ้าง)
-3. นางสาวธนพัฒน์ บุญช่วย (25–44 ปี, พนักงานบริษัท)
-4. นายธนวัฒน์ บุญช่วย (25–44 ปี, รับจ้าง)
-5. เด็กชายชัชธนนฌ์ วโรธรวัช (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางบุญเรือง พรมทัศน์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)
+2. นางสาวมยุรีย์ พรมทัศน์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)
+3. นางสาวธนพัฒน์ บุญช่วย (หญิง, 25–44 ปี, พนักงานบริษัท)
+4. นายธนวัฒน์ บุญช่วย (ชาย, 25–44 ปี, รับจ้าง)
+5. เด็กชายชัชธนนฌ์ วโรธรวัช (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G19" s="4" t="n">
@@ -2200,8 +2200,8 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>1. สมหมาย หนูเกต (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายศุทินันท์ หนูเกต (25–44 ปี, รับจ้าง)</t>
+          <t>1. สมหมาย หนูเกต (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายศุทินันท์ หนูเกต (ชาย, 25–44 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวมาลัย องคศิลป์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวมาลัย องคศิลป์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G21" s="4" t="n">
@@ -2373,8 +2373,8 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>1. นายบรรจง บุญรอด (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสาวพรพิมล พูนศิริ (25–44 ปี, พยาบาล)</t>
+          <t>1. นายบรรจง บุญรอด (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางสาวพรพิมล พูนศิริ (หญิง, 25–44 ปี, พยาบาล)</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
@@ -2460,10 +2460,10 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>1. สังวาลย์ สุขสว่าง (60 ปีขึ้นไป, รับจ้าง)
-2. สมหวัง สุขสว่าง (25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. ภาคภูมิ สุขสว่าง (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-4. พีรพล สุขสว่าง (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. สังวาลย์ สุขสว่าง (หญิง, 60 ปีขึ้นไป, รับจ้าง)
+2. สมหวัง สุขสว่าง (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. ภาคภูมิ สุขสว่าง (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
+4. พีรพล สุขสว่าง (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
@@ -2549,9 +2549,9 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>1. นางสาวสาวินีย์ สีกาสี (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายอิงอร โม่ไหม (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. เด็กหญิงสรินพร โม่ไหม (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางสาวสาวินีย์ สีกาสี (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายอิงอร โม่ไหม (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. เด็กหญิงสรินพร โม่ไหม (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>1. นางประยงค์ พรหมทัศน์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางประยงค์ พรหมทัศน์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G25" s="4" t="n">
@@ -2723,8 +2723,8 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>1. นายประวิทย์ บุญช่วย (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางบุญยืน บุญช่วย (60 ปีขึ้นไป, อสม)</t>
+          <t>1. นายประวิทย์ บุญช่วย (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางบุญยืน บุญช่วย (หญิง, 60 ปีขึ้นไป, อสม)</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
@@ -2810,8 +2810,8 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>1. นายสมคิด เวียงสมุทร (60 ปีขึ้นไป, เกษตรกรรม)
-2. นางส้มเกลี้ยง เวียงสมุทร (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายสมคิด เวียงสมุทร (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+2. นางส้มเกลี้ยง เวียงสมุทร (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G27" s="4" t="n">
@@ -2897,11 +2897,11 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>1. นภา สวนรักษา (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. คำรณค์ สวนรักษา (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. นพดล สวนรักษา (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-4. พงษกรณ์ สวนรักษา (15–24 ปี, นักเรียน/นักศึกษา)
-5. ภรกรณ์ สวนรักษา (15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นภา สวนรักษา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. คำรณค์ สวนรักษา (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. นพดล สวนรักษา (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+4. พงษกรณ์ สวนรักษา (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)
+5. ภรกรณ์ สวนรักษา (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
@@ -2987,10 +2987,10 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>1. นางอ้อย อยู่สุข (60 ปีขึ้นไป, เกษตรกรรม)
-2. นายรุ่ง ปามา (60 ปีขึ้นไป, รับจ้าง)
-3. นายธีรภัทร พรหมพัฒน์ (15–24 ปี, รับจ้าง)
-4. นางสาววัชนี พรหมพัฒน์ (15–24 ปี, รับจ้าง)</t>
+          <t>1. นางอ้อย อยู่สุข (หญิง, 60 ปีขึ้นไป, เกษตรกรรม)
+2. นายรุ่ง ปามา (ชาย, 60 ปีขึ้นไป, รับจ้าง)
+3. นายธีรภัทร พรหมพัฒน์ (ชาย, 15–24 ปี, รับจ้าง)
+4. นางสาววัชนี พรหมพัฒน์ (หญิง, 15–24 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G29" s="4" t="n">
@@ -3076,9 +3076,9 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>1. ไพทูรย์ โชคชัยฤทธิ์ (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ปทุม เมฆจั่น (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. พลอยรัตน์ โชคชัยฤทธิ์ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. ไพทูรย์ โชคชัยฤทธิ์ (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. ปทุม เมฆจั่น (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+3. พลอยรัตน์ โชคชัยฤทธิ์ (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวอรนุช คุ้มทรัพย์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวอรนุช คุ้มทรัพย์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G31" s="4" t="n">
@@ -3250,8 +3250,8 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>1. นายประเสริฐ เกศมาลา (60 ปีขึ้นไป, ได้รายได้จากลูกชาย)
-2. นางนางใจ เกศมาลา (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายประเสริฐ เกศมาลา (ชาย, 60 ปีขึ้นไป, ได้รายได้จากลูกชาย)
+2. นางนางใจ เกศมาลา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>1. นาวสำรวย คงผงแผ้ว (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นาวสำรวย คงผงแผ้ว (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G33" s="4" t="n">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>1. ภัทรทาดา ทองคำ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ภัทรทาดา ทองคำ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
@@ -3509,8 +3509,8 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>1. นายมนตรี มนต์คจรเดชา (60 ปีขึ้นไป, เกษตรกรรม)
-2. นางมาลี มนต์คจรเดชา (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายมนตรี มนต์คจรเดชา (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+2. นางมาลี มนต์คจรเดชา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G35" s="4" t="n">
@@ -3596,8 +3596,8 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>1. นายโฉม ชัยศรีเกษมพันธุ์ (60 ปีขึ้นไป, เกษตรกรรม)
-2. นางลำเพย ชัยศรีเกษมพันธุ์ (60 ปีขึ้นไป, รับจ้าง)</t>
+          <t>1. นายโฉม ชัยศรีเกษมพันธุ์ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+2. นางลำเพย ชัยศรีเกษมพันธุ์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
@@ -3683,12 +3683,12 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>1. ลภัสลดา ผู้ทัด (45–59 ปี, ไม่ได้ประกอบอาชีพ)
-2. สาลี่ บุญรอด (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. อภิวัฒน์ ผู้ทัด (15–24 ปี, รับจ้าง)
-4. รัตนาภร อเนก (15–24 ปี, รับจ้าง)
-5. ภิรมย์ ผู้ทัด (45–59 ปี, รับจ้าง)
-6. พราวณิรินทร์ ผู้ทัด (ต่ำกว่า 15 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ลภัสลดา ผู้ทัด (หญิง, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
+2. สาลี่ บุญรอด (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. อภิวัฒน์ ผู้ทัด (ชาย, 15–24 ปี, รับจ้าง)
+4. รัตนาภร อเนก (หญิง, 15–24 ปี, รับจ้าง)
+5. ภิรมย์ ผู้ทัด (ชาย, 45–59 ปี, รับจ้าง)
+6. พราวณิรินทร์ ผู้ทัด (หญิง, ต่ำกว่า 15 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G37" s="4" t="n">
@@ -3774,8 +3774,8 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>1. สนอง ทองคำ (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. สุขสันต์ เลิศรัตน์ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. สนอง ทองคำ (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. สุขสันต์ เลิศรัตน์ (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
@@ -3861,10 +3861,10 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>1. ธัญพร บุญรอด (45–59 ปี, รายได้จากสามี)
-2. ณัฐพล อรวีรนนท์ (45–59 ปี, ขับแท็กซี่)
-3. อุทัย บุญรอด (45–59 ปี, ไม่ได้ประกอบอาชีพ)
-4. สุดารัตน์ บุญรอด (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ธัญพร บุญรอด (หญิง, 45–59 ปี, รายได้จากสามี)
+2. ณัฐพล อรวีรนนท์ (ชาย, 45–59 ปี, ขับแท็กซี่)
+3. อุทัย บุญรอด (ชาย, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
+4. สุดารัตน์ บุญรอด (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G39" s="4" t="n">
@@ -3950,9 +3950,9 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>1. นางเสาวลักษณ์ พูนศิริ (25–44 ปี, พนักงานบริษัท)
-2. ด.ญ.วิไลลักษณ์ พูนศิริ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-3. ด.ญ.วิลัยวรรณ พูนศิริ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางเสาวลักษณ์ พูนศิริ (หญิง, 25–44 ปี, พนักงานบริษัท)
+2. ด.ญ.วิไลลักษณ์ พูนศิริ (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
+3. ด.ญ.วิลัยวรรณ พูนศิริ (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
@@ -4038,9 +4038,9 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>1. นางสุริยา กองประเสริฐ (60 ปีขึ้นไป, เกษตรกรรม)
-2. นายกรวิช กองประเสริฐ (60 ปีขึ้นไป, เกษตรกรรม)
-3. นางสาวเขมมิกา กองประเสริฐ (25–44 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
+          <t>1. นางสุริยา กองประเสริฐ (หญิง, 60 ปีขึ้นไป, เกษตรกรรม)
+2. นายกรวิช กองประเสริฐ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+3. นางสาวเขมมิกา กองประเสริฐ (หญิง, 25–44 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
         </is>
       </c>
       <c r="G41" s="4" t="n">
@@ -4126,8 +4126,8 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>1. ทองสุข บุญธรรม (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. บุญลือ บุญธรรม (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ทองสุข บุญธรรม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. บุญลือ บุญธรรม (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>1. ไพศล ทองพูน (45–59 ปี, รับจ้าง)</t>
+          <t>1. ไพศล ทองพูน (ชาย, 45–59 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G43" s="4" t="n">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>1. นางบังอ้อย พิษณุนาวิน (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นายจำเลียง บุญมี (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นางวันเพ็ญ ขันเงิน (25–44 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. ด.ช.ณัฐพัฒน์ สันเงิน (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-5. ด.ช.ภูมิพัฒน์ ขันเงิน (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางบังอ้อย พิษณุนาวิน (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นายจำเลียง บุญมี (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นางวันเพ็ญ ขันเงิน (หญิง, 25–44 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. ด.ช.ณัฐพัฒน์ สันเงิน (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
+5. ด.ช.ภูมิพัฒน์ ขันเงิน (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>1. มานัด ทองพูน (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. มานัด ทองพูน (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G45" s="4" t="n">
@@ -4475,10 +4475,10 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>1. บุญเลิศ ทองคำ (60 ปีขึ้นไป, เกษตรกรรม)
-2. อนงค์ ทองคำ (60 ปีขึ้นไป, เกษตรกรรม)
-3. อนุสิทธิ์ ทองคำ (15–24 ปี, นักเรียน/นักศึกษา)
-4. เต็มวุฒิ ทองคำ (15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. บุญเลิศ ทองคำ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+2. อนงค์ ทองคำ (หญิง, 60 ปีขึ้นไป, เกษตรกรรม)
+3. อนุสิทธิ์ ทองคำ (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)
+4. เต็มวุฒิ ทองคำ (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
@@ -4564,9 +4564,9 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>1. นางอำพร รุ่งสว่าง (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางจริญ จิราวัฒ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายชูเกียรติ สมรักษา (25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. นางอำพร รุ่งสว่าง (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางจริญ จิราวัฒ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายชูเกียรติ สมรักษา (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G47" s="4" t="n">
@@ -4652,8 +4652,8 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>1. ไพเราะ มนต์ขจรเดชา (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ปรีชา บุญธรรม (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ไพเราะ มนต์ขจรเดชา (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. ปรีชา บุญธรรม (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
@@ -4739,10 +4739,10 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>1. ปราโมทย์ รื่นรวย (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. สมหมาย รื่นรวย (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. สมมาตร รื่นรวย (25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-4. กิตติมา รื่นรวย (25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ปราโมทย์ รื่นรวย (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. สมหมาย รื่นรวย (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+3. สมมาตร รื่นรวย (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+4. กิตติมา รื่นรวย (หญิง, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G49" s="4" t="n">
@@ -4828,8 +4828,8 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>1. พรจิตร ทองสนธิ (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ฉัตรชัย ประสงค์เงิน (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. พรจิตร ทองสนธิ (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. ฉัตรชัย ประสงค์เงิน (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
@@ -4915,9 +4915,9 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>1. ลินนา ตันพาณิชย์ (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. วัฒนา บุญมี (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. วรพจน์ บุญมี (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ลินนา ตันพาณิชย์ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. วัฒนา บุญมี (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+3. วรพจน์ บุญมี (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G51" s="4" t="n">
@@ -5003,10 +5003,10 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>1. วันเพ็ญ บุญรอด (60 ปีขึ้นไป, ข้าราชการบำนาญ)
-2. บรรเจิด บุญรอด (60 ปีขึ้นไป, ข้าราชการบำนาญ)
-3. วงศกร บุญรอด (60 ปีขึ้นไป, พนักงานบริษัท)
-4. วีรากร บุญรอด (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. วันเพ็ญ บุญรอด (หญิง, 60 ปีขึ้นไป, ข้าราชการบำนาญ)
+2. บรรเจิด บุญรอด (ชาย, 60 ปีขึ้นไป, ข้าราชการบำนาญ)
+3. วงศกร บุญรอด (ชาย, 60 ปีขึ้นไป, พนักงานบริษัท)
+4. วีรากร บุญรอด (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
@@ -5092,12 +5092,12 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>1. นายประจวบ ทองสนธิ (60 ปีขึ้นไป, รับจ้าง)
-2. นางพุทธชาติ ทองสนธิ (45–59 ปี, แม่บ้าน)
-3. นายทศพล ทองสนธิ (25–44 ปี, รับจ้าง)
-4. นายสกล ทองสนธิ (25–44 ปี, รับจ้าง)
-5. ด.ช.จักรกฤษณ์ ทองสนธิ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-6. ด.ช.ภพพิพัฒน์ ทองสนธิ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นายประจวบ ทองสนธิ (ชาย, 60 ปีขึ้นไป, รับจ้าง)
+2. นางพุทธชาติ ทองสนธิ (หญิง, 45–59 ปี, แม่บ้าน)
+3. นายทศพล ทองสนธิ (ชาย, 25–44 ปี, รับจ้าง)
+4. นายสกล ทองสนธิ (ชาย, 25–44 ปี, รับจ้าง)
+5. ด.ช.จักรกฤษณ์ ทองสนธิ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
+6. ด.ช.ภพพิพัฒน์ ทองสนธิ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G53" s="4" t="n">
@@ -5183,8 +5183,8 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>1. ศิริญญา รื่นรวย (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. ณปภากร สุขพงศ์ไทย (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. ศิริญญา รื่นรวย (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. ณปภากร สุขพงศ์ไทย (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
@@ -5270,11 +5270,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>1. นายมงคล พลอยสมุทร (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางอรอุษา พลอยสมุทร (45–59 ปี, รับจ้าง)
-3. นางสาวนฤมล พลอยสมุทร (25–44 ปี, พนักงานบริษัท)
-4. นายอดิศร พลอยสมุทร (25–44 ปี, ช่างไฟฟ้า)
-5. ด.ญ.นฐพร พลอยสมุทร (ต่ำกว่า 15 ปี, ยังไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายมงคล พลอยสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางอรอุษา พลอยสมุทร (หญิง, 45–59 ปี, รับจ้าง)
+3. นางสาวนฤมล พลอยสมุทร (หญิง, 25–44 ปี, พนักงานบริษัท)
+4. นายอดิศร พลอยสมุทร (ชาย, 25–44 ปี, ช่างไฟฟ้า)
+5. ด.ญ.นฐพร พลอยสมุทร (หญิง, ต่ำกว่า 15 ปี, ยังไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G55" s="4" t="n">
@@ -5360,9 +5360,9 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>1. จำเนียร รัศมี (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. ปัญญารัตน์ รัศมี (45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-3. มาโนช นาคก่ำ (45–59 ปี, เกษตรกรรม)</t>
+          <t>1. จำเนียร รัศมี (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. ปัญญารัตน์ รัศมี (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
+3. มาโนช นาคก่ำ (ชาย, 45–59 ปี, เกษตรกรรม)</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
@@ -5448,11 +5448,11 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวดาราวรรณ ละมั่งทอง (60 ปีขึ้นไป, พนักงานบริษัท)
-2. นางสาวรัศมี เกตุแก้ว (15–24 ปี, พนักงานบริษัท)
-3. ด.ช.เตชินท์ ละมั่งทอง (ต่ำกว่า 15 ปี, แรกเกิด)
-4. นายพีระวัฒน์ วงค์นิล (25–44 ปี, พนักงานบริษัท)
-5. นายธยธร เนียมชาติ (25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวดาราวรรณ ละมั่งทอง (หญิง, 60 ปีขึ้นไป, พนักงานบริษัท)
+2. นางสาวรัศมี เกตุแก้ว (หญิง, 15–24 ปี, พนักงานบริษัท)
+3. ด.ช.เตชินท์ ละมั่งทอง (ชาย, ต่ำกว่า 15 ปี, แรกเกิด)
+4. นายพีระวัฒน์ วงค์นิล (ชาย, 25–44 ปี, พนักงานบริษัท)
+5. นายธยธร เนียมชาติ (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G57" s="4" t="n">
@@ -5538,8 +5538,8 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>1. สมร จันทร์ทร (60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ภิญญาธิดา มลขจรเดชา (15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. สมร จันทร์ทร (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
+2. ภิญญาธิดา มลขจรเดชา (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>1. มะลิวรรณ ชีวงษ์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. มะลิวรรณ ชีวงษ์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G59" s="4" t="n">
@@ -5711,8 +5711,8 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>1. สนธยา จันทร์ทร (60 ปีขึ้นไป, เกษตรกรรม)
-2. ณัฐกร จันทร์ทร (15–24 ปี, รับจ้าง)</t>
+          <t>1. สนธยา จันทร์ทร (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
+2. ณัฐกร จันทร์ทร (ชาย, 15–24 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
@@ -5798,9 +5798,9 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>1. ชวลิต รื่นเริง (45–59 ปี, รับจ้าง)
-2. ลัดดา ชีวงษ์ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. ภาคภูมิ รื่นเริง (45–59 ปี, รับจ้าง)</t>
+          <t>1. ชวลิต รื่นเริง (ชาย, 45–59 ปี, รับจ้าง)
+2. ลัดดา ชีวงษ์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. ภาคภูมิ รื่นเริง (ชาย, 45–59 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G61" s="4" t="n">
@@ -5886,8 +5886,8 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>1. อนุชา เพชรชะรัด (45–59 ปี, รับจ้าง)
-2. ทองอยู่ เพชรชะรัด (60 ปีขึ้นไป, รับจ้าง)</t>
+          <t>1. อนุชา เพชรชะรัด (ชาย, 45–59 ปี, รับจ้าง)
+2. ทองอยู่ เพชรชะรัด (ชาย, 60 ปีขึ้นไป, รับจ้าง)</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
@@ -5973,9 +5973,9 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>1. นางบุญลือ จิตรวัฒน์ (60 ปีขึ้นไป, รับจ้าง)
-2. นายขวัญชัย ทองรัศมี (45–59 ปี, รับจ้าง)
-3. นายธีรศักศ์ ทองรัศมี (15–24 ปี, รับจ้าง)</t>
+          <t>1. นางบุญลือ จิตรวัฒน์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)
+2. นายขวัญชัย ทองรัศมี (ชาย, 45–59 ปี, รับจ้าง)
+3. นายธีรศักศ์ ทองรัศมี (ชาย, 15–24 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G63" s="4" t="n">
@@ -6061,7 +6061,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>1. นางอิ่ม ภักดีคำ (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางอิ่ม ภักดีคำ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
@@ -6147,10 +6147,10 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>1. นางสมศรี แซ่ฮั่ง (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายขจรศักดิ์ ฉั่วยู่เน้ย (25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. นางสาวกุลธิชา พุทธม้าสี (25–44 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. นายอนุชา ฉั่วยู่เน้ย (25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสมศรี แซ่ฮั่ง (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายขจรศักดิ์ ฉั่วยู่เน้ย (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. นางสาวกุลธิชา พุทธม้าสี (หญิง, 25–44 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. นายอนุชา ฉั่วยู่เน้ย (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G65" s="4" t="n">
@@ -6236,9 +6236,9 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>1. นายทศกร ทองชาวนา (45–59 ปี, รับจ้าง)
-2. นางสาวกมลพร พัคดีธรรม (45–59 ปี, พนักงานบริษัท)
-3. นายธีรการ ทองชาวนา (15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นายทศกร ทองชาวนา (ชาย, 45–59 ปี, รับจ้าง)
+2. นางสาวกมลพร พัคดีธรรม (หญิง, 45–59 ปี, พนักงานบริษัท)
+3. นายธีรการ ทองชาวนา (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
@@ -6324,10 +6324,10 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>1. สุจินดา เกาะประเสริฐ (45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-2. กรทิพย์ เกาะประเสริฐ (25–44 ปี, ผู้ช่วยผู้ใหญ่บ้าน)
-3. ชิษณุพงษ์ เกาะประเสริฐ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-4. ระพีพงษ์ เกาะประเสริฐ (ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. สุจินดา เกาะประเสริฐ (ชาย, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
+2. กรทิพย์ เกาะประเสริฐ (หญิง, 25–44 ปี, ผู้ช่วยผู้ใหญ่บ้าน)
+3. ชิษณุพงษ์ เกาะประเสริฐ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
+4. ระพีพงษ์ เกาะประเสริฐ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G67" s="4" t="n">
@@ -6413,7 +6413,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>1. ธงชัย โชคชัยฤทธิ์ (60 ปีขึ้นไป, เกษตรกรรม)</t>
+          <t>1. ธงชัย โชคชัยฤทธิ์ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
@@ -6499,12 +6499,12 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>1. นางพยอม เขียวสมุทร (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นายโสภา เขียวสมุทร (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายธีระยุทธ์ เขียวสมุทร (45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-4. นางกนกกร เขียวสมุทร (25–44 ปี, อสม)
-5. นายชวกร เขียวสมุทร (15–24 ปี, เรียนอยู่)
-6. นางสาวมณีรัตน์ เขียวสมุทร (25–44 ปี, เรียนอยู่)</t>
+          <t>1. นางพยอม เขียวสมุทร (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นายโสภา เขียวสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายธีระยุทธ์ เขียวสมุทร (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+4. นางกนกกร เขียวสมุทร (หญิง, 25–44 ปี, อสม)
+5. นายชวกร เขียวสมุทร (ชาย, 15–24 ปี, เรียนอยู่)
+6. นางสาวมณีรัตน์ เขียวสมุทร (หญิง, 25–44 ปี, เรียนอยู่)</t>
         </is>
       </c>
       <c r="G69" s="4" t="n">
@@ -6590,12 +6590,12 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>1. นายสันต์ รัศมี (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสำลี รัศมี (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายสุรชัย รัศมี (45–59 ปี, ไม่ได้ประกอบอาชีพ)
-4. นายอนพัฒน์ รัศมี (15–24 ปี, พนักงานบริษัท)
-5. นายสุพัฒน์ รัศมี (15–24 ปี, พนักงานบริษัท)
-6. นางสาววศิตา  เจ๊ะอาแส (25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายสันต์ รัศมี (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางสำลี รัศมี (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+3. นายสุรชัย รัศมี (ชาย, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
+4. นายอนพัฒน์ รัศมี (ชาย, 15–24 ปี, พนักงานบริษัท)
+5. นายสุพัฒน์ รัศมี (ชาย, 15–24 ปี, พนักงานบริษัท)
+6. นางสาววศิตา  เจ๊ะอาแส (หญิง, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
@@ -6681,7 +6681,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>1. ขวัญใจ ชื่นชม (60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ขวัญใจ ชื่นชม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G71" s="4" t="n">
@@ -14294,7 +14294,11 @@
           <t>เด็กหญิงสรินพร โม่ไหม</t>
         </is>
       </c>
-      <c r="E70" s="6" t="inlineStr"/>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>หญิง</t>
+        </is>
+      </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
           <t>ต่ำกว่า 15 ปี</t>
@@ -15190,7 +15194,11 @@
           <t>นพดล สวนรักษา</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr"/>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>ชาย</t>
+        </is>
+      </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
           <t>45–59 ปี</t>

</xml_diff>

<commit_message>
Correct 4 female members gender: Female 97, Male 107, update downloadable excel
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -618,7 +618,7 @@
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>1. นางสาวเพ็ญนภา บุญเสริม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางราวี เวียงสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางราวี เวียงสมุทร (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
 3. นายถาวร เวียงสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
 4. นางภิรมณ์พร บุญจันที (หญิง, 45–59 ปี, ครูผู้ช่วย)
 5. นางสาวกัญญารัตน์ อัมไพ (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
@@ -796,7 +796,7 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>1. นายทองคำ เลิศพาณุมาศ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสุมาลี พวงโคสน (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางสุมาลี พวงโคสน (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
 3. นายประสิทธิ์ เลิศพาณุมาศ (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)
 4. ด.ช.ปนชัย เลิศพาณุมาศ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
@@ -1060,7 +1060,7 @@
       <c r="F7" s="5" t="inlineStr">
         <is>
           <t>1. นายนุกุล อยู่สุข (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นางนงนุช อยู่สุข (ชาย, 45–59 ปี, เกษตรกรรม)
+2. นางนงนุช อยู่สุข (หญิง, 45–59 ปี, เกษตรกรรม)
 3. นายธนดล อยู่สุข (ชาย, 25–44 ปี, เกษตรกรรม)
 4. นางวรัญธร อยู่สุข (หญิง, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
@@ -1500,7 +1500,7 @@
       <c r="F12" s="3" t="inlineStr">
         <is>
           <t>1. นายถวัลย์ คำประสิทธิ์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางไพรัตน์ คำประสิทธิ์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
+2. นางไพรัตน์ คำประสิทธิ์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
 3. นายกิตติพงศ์ คำประสิทธิ์ (ชาย, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
 4. นายพงศธร คำประสิทธิ์ (ชาย, 45–59 ปี, รับจ้าง)
 5. นางกมลรัตน์ คำประสิทธิ์ (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>ชาย</t>
+          <t>หญิง</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -7910,7 +7910,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>ชาย</t>
+          <t>หญิง</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>ชาย</t>
+          <t>หญิง</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>ชาย</t>
+          <t>หญิง</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Update BMI data to N=204 with complete records in dashboard and excel
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -479,7 +479,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="31.6" customWidth="1" min="2" max="2"/>
@@ -6755,7 +6755,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X205"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.7" customWidth="1" min="1" max="1"/>
     <col width="31.6" customWidth="1" min="2" max="2"/>
@@ -7920,22 +7920,22 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>52</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>152</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22.5</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -8424,12 +8424,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>23:4</t>
+          <t>23.4</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ท้วม (น้ำหนักเกิน)</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
@@ -12148,12 +12148,24 @@
           <t>60 ปีขึ้นไป</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr"/>
-      <c r="H50" s="7" t="inlineStr"/>
-      <c r="I50" s="6" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>22.8</t>
+        </is>
+      </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr">
@@ -12246,12 +12258,24 @@
           <t>45–59 ปี</t>
         </is>
       </c>
-      <c r="G51" s="9" t="inlineStr"/>
-      <c r="H51" s="9" t="inlineStr"/>
-      <c r="I51" s="8" t="inlineStr"/>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>24.1</t>
+        </is>
+      </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ท้วม (น้ำหนักเกิน)</t>
         </is>
       </c>
       <c r="K51" s="9" t="inlineStr">
@@ -12344,12 +12368,24 @@
           <t>60 ปีขึ้นไป</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr"/>
-      <c r="H52" s="7" t="inlineStr"/>
-      <c r="I52" s="6" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>162</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>21.0</t>
+        </is>
+      </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
@@ -15630,22 +15666,22 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>58</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>164</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21.6</t>
         </is>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K82" s="7" t="inlineStr">
@@ -17684,7 +17720,7 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>65</t>
         </is>
       </c>
       <c r="H101" s="9" t="inlineStr">
@@ -17694,12 +17730,12 @@
       </c>
       <c r="I101" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="J101" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ท้วม (น้ำหนักเกิน)</t>
         </is>
       </c>
       <c r="K101" s="9" t="inlineStr">
@@ -19718,22 +19754,22 @@
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>53</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>156</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21.8</t>
         </is>
       </c>
       <c r="J120" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K120" s="7" t="inlineStr">
@@ -19832,22 +19868,22 @@
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32</t>
         </is>
       </c>
       <c r="H121" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>138</t>
         </is>
       </c>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16.8</t>
         </is>
       </c>
       <c r="J121" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>น้ำหนักน้อย (ผอม)</t>
         </is>
       </c>
       <c r="K121" s="9" t="inlineStr">
@@ -19938,22 +19974,22 @@
       </c>
       <c r="G122" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25</t>
         </is>
       </c>
       <c r="H122" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>125</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="J122" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>น้ำหนักน้อย (ผอม)</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr">
@@ -22622,7 +22658,7 @@
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>64</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
@@ -22632,12 +22668,12 @@
       </c>
       <c r="I146" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22.1</t>
         </is>
       </c>
       <c r="J146" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K146" s="7" t="inlineStr">
@@ -22842,22 +22878,22 @@
       </c>
       <c r="G148" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>68</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>172</t>
         </is>
       </c>
       <c r="I148" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="J148" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ท้วม (น้ำหนักเกิน)</t>
         </is>
       </c>
       <c r="K148" s="7" t="inlineStr">
@@ -22948,7 +22984,7 @@
       </c>
       <c r="G149" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H149" s="9" t="inlineStr">
@@ -22958,12 +22994,12 @@
       </c>
       <c r="I149" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22.2</t>
         </is>
       </c>
       <c r="J149" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K149" s="9" t="inlineStr">
@@ -23164,22 +23200,22 @@
       </c>
       <c r="G151" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H151" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>130</t>
         </is>
       </c>
       <c r="I151" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16.6</t>
         </is>
       </c>
       <c r="J151" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>น้ำหนักน้อย (ผอม)</t>
         </is>
       </c>
       <c r="K151" s="9" t="inlineStr">
@@ -24599,17 +24635,17 @@
       </c>
       <c r="H164" s="7" t="inlineStr">
         <is>
-          <t>ผ58</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I164" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="J164" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>น้ำหนักน้อย (ผอม)</t>
         </is>
       </c>
       <c r="K164" s="7" t="inlineStr">
@@ -25024,12 +25060,24 @@
           <t>15–24 ปี</t>
         </is>
       </c>
-      <c r="G168" s="7" t="inlineStr"/>
-      <c r="H168" s="7" t="inlineStr"/>
-      <c r="I168" s="6" t="inlineStr"/>
+      <c r="G168" s="7" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="H168" s="7" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="I168" s="6" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
       <c r="J168" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>สมส่วน (ปกติ)</t>
         </is>
       </c>
       <c r="K168" s="7" t="inlineStr">
@@ -25628,12 +25676,24 @@
           <t>45–59 ปี</t>
         </is>
       </c>
-      <c r="G174" s="7" t="inlineStr"/>
-      <c r="H174" s="7" t="inlineStr"/>
-      <c r="I174" s="6" t="inlineStr"/>
+      <c r="G174" s="7" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="H174" s="7" t="inlineStr">
+        <is>
+          <t>168</t>
+        </is>
+      </c>
+      <c r="I174" s="6" t="inlineStr">
+        <is>
+          <t>23.4</t>
+        </is>
+      </c>
       <c r="J174" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ท้วม (น้ำหนักเกิน)</t>
         </is>
       </c>
       <c r="K174" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Update BMI to include only age >= 15 (N=184)
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -6766,7 +6766,7 @@
     <col width="19.9" customWidth="1" min="7" max="7"/>
     <col width="19.9" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="26.4" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
     <col width="23.8" customWidth="1" min="11" max="11"/>
     <col width="30.3" customWidth="1" min="12" max="12"/>
     <col width="26.4" customWidth="1" min="13" max="13"/>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ภาวะโภชนาการ</t>
+          <t>ภาวะโภชนาการ (เกณฑ์ผู้ใหญ่ 15 ปีขึ้นไป)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -7710,12 +7710,12 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>21.4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -8122,12 +8122,12 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>20.76</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
@@ -13060,12 +13060,12 @@
       </c>
       <c r="I58" s="6" t="inlineStr">
         <is>
-          <t>19.32</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K58" s="7" t="inlineStr">
@@ -13920,12 +13920,12 @@
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>15.31</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr">
@@ -14026,12 +14026,12 @@
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J67" s="8" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K67" s="9" t="inlineStr">
@@ -14352,12 +14352,12 @@
       </c>
       <c r="I70" s="6" t="inlineStr">
         <is>
-          <t>15.4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K70" s="7" t="inlineStr">
@@ -16162,12 +16162,12 @@
       </c>
       <c r="I87" s="8" t="inlineStr">
         <is>
-          <t>14.29</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K87" s="9" t="inlineStr">
@@ -17808,12 +17808,12 @@
       </c>
       <c r="I102" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K102" s="7" t="inlineStr">
@@ -18672,12 +18672,12 @@
       </c>
       <c r="I110" s="6" t="inlineStr">
         <is>
-          <t>14.79</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J110" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K110" s="7" t="inlineStr">
@@ -18774,12 +18774,12 @@
       </c>
       <c r="I111" s="8" t="inlineStr">
         <is>
-          <t>15.12</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J111" s="8" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K111" s="9" t="inlineStr">
@@ -19878,12 +19878,12 @@
       </c>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>16.8</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J121" s="8" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K121" s="9" t="inlineStr">
@@ -19984,12 +19984,12 @@
       </c>
       <c r="I122" s="6" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J122" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr">
@@ -22558,12 +22558,12 @@
       </c>
       <c r="I145" s="8" t="inlineStr">
         <is>
-          <t>18.6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J145" s="8" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K145" s="9" t="inlineStr">
@@ -23100,12 +23100,12 @@
       </c>
       <c r="I150" s="6" t="inlineStr">
         <is>
-          <t>19.53</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J150" s="6" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K150" s="7" t="inlineStr">
@@ -23210,12 +23210,12 @@
       </c>
       <c r="I151" s="8" t="inlineStr">
         <is>
-          <t>16.6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J151" s="8" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K151" s="9" t="inlineStr">
@@ -23430,12 +23430,12 @@
       </c>
       <c r="I153" s="8" t="inlineStr">
         <is>
-          <t>19.02</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J153" s="8" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K153" s="9" t="inlineStr">
@@ -23980,12 +23980,12 @@
       </c>
       <c r="I158" s="6" t="inlineStr">
         <is>
-          <t>17.19</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J158" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K158" s="7" t="inlineStr">
@@ -24640,12 +24640,12 @@
       </c>
       <c r="I164" s="6" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J164" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K164" s="7" t="inlineStr">
@@ -27392,12 +27392,12 @@
       </c>
       <c r="I190" s="6" t="inlineStr">
         <is>
-          <t>16.44</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J190" s="6" t="inlineStr">
         <is>
-          <t>น้ำหนักน้อย (ผอม)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K190" s="7" t="inlineStr">
@@ -27486,12 +27486,12 @@
       </c>
       <c r="I191" s="8" t="inlineStr">
         <is>
-          <t>20.36</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J191" s="8" t="inlineStr">
         <is>
-          <t>สมส่วน (ปกติ)</t>
+          <t>&lt; 15 ปี (ไม่ประเมิน BMI ผู้ใหญ่)</t>
         </is>
       </c>
       <c r="K191" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Add Dietary Habits slide (N=70 households) and update Excel
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:S71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -491,14 +491,15 @@
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="34.2" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
     <col width="34.2" customWidth="1" min="12" max="12"/>
-    <col width="21.2" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="34.2" customWidth="1" min="13" max="13"/>
+    <col width="21.2" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
     <col width="45" customWidth="1" min="17" max="17"/>
-    <col width="17.3" customWidth="1" min="18" max="18"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="17.3" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -554,40 +555,45 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>พฤติกรรมบริโภค (โซเดียม/น้ำตาล/น้ำมัน)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>สภาพภายในบ้าน</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>สภาพรอบบ้าน</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>การระบายอากาศ</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>แสงสว่าง</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ปัญหาฝุ่น/ควัน/กลิ่น</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>การจัดการขยะ</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>การกำจัดน้ำเสีย</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>สัตว์เลี้ยง</t>
         </is>
@@ -644,40 +650,47 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(รถตามถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>ฝังกลบ, อบต./เทศบาลมาเก็บ, ทิ้งลงแม่น้ำ/ลำคลอง</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน, บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -732,40 +745,47 @@
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -821,40 +841,47 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -909,40 +936,47 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(เสียงรถบริเวณถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q5" s="5" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -996,40 +1030,47 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(รถสัญจรไปมา)</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="S6" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1085,40 +1126,47 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O7" s="5" t="inlineStr">
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr">
+      <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q7" s="5" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr">
+      <c r="S7" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1173,40 +1221,47 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(มีเสียงรถตามถนน), กลิ่น(มี (จากขยะ), คูน้ำหลังบ้านซึ่งชาวบ้านปล่อยน้ำจากบ่อกุ้ง)</t>
         </is>
       </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="inlineStr">
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>คูน้ำหลังบ้าน</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
+      <c r="S8" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -1261,40 +1316,47 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>ไม่เพียงพอ</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(เสียงจากรถมอเตอร์ไซค์), กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P9" s="5" t="inlineStr">
+      <c r="Q9" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q9" s="5" t="inlineStr">
+      <c r="R9" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R9" s="5" t="inlineStr">
+      <c r="S9" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1350,40 +1412,47 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q10" s="3" t="inlineStr">
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>เทลงคูน้ำตอนน้ำทะเลหนุน</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
+      <c r="S10" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1436,40 +1505,47 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O11" s="5" t="inlineStr">
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(เสียงรถตามถนน), กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P11" s="5" t="inlineStr">
+      <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>ฝังกลบ</t>
         </is>
       </c>
-      <c r="Q11" s="5" t="inlineStr">
+      <c r="R11" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R11" s="5" t="inlineStr">
+      <c r="S11" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1526,40 +1602,47 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(การสัญจรรถ และเสียงรถแต่ง)</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q12" s="3" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R12" s="3" t="inlineStr">
+      <c r="S12" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1613,40 +1696,47 @@
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O13" s="5" t="inlineStr">
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P13" s="5" t="inlineStr">
+      <c r="Q13" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q13" s="5" t="inlineStr">
+      <c r="R13" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R13" s="5" t="inlineStr">
+      <c r="S13" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1699,40 +1789,47 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="R14" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
+      <c r="S14" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -1787,40 +1884,47 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O15" s="5" t="inlineStr">
+      <c r="P15" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(เสียงรถตามถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P15" s="5" t="inlineStr">
+      <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q15" s="5" t="inlineStr">
+      <c r="R15" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1872,40 +1976,47 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>ไม่เพียงพอ</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="R16" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R16" s="3" t="inlineStr">
+      <c r="S16" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -1961,40 +2072,47 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="M17" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O17" s="5" t="inlineStr">
+      <c r="P17" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(รถสัญจรไปมา)</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr">
+      <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q17" s="5" t="inlineStr">
+      <c r="R17" s="5" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R17" s="5" t="inlineStr">
+      <c r="S17" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -2047,40 +2165,47 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q18" s="3" t="inlineStr">
+      <c r="R18" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R18" s="3" t="inlineStr">
+      <c r="S18" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -2137,40 +2262,47 @@
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="M19" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="O19" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O19" s="5" t="inlineStr">
+      <c r="P19" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P19" s="5" t="inlineStr">
+      <c r="Q19" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q19" s="5" t="inlineStr">
+      <c r="R19" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R19" s="5" t="inlineStr">
+      <c r="S19" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -2224,40 +2356,47 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(รถยนต์ตามถนน สุนัข), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q20" s="3" t="inlineStr">
+      <c r="R20" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน, ทิ้งในคลองหลังบ้าน</t>
         </is>
       </c>
-      <c r="R20" s="3" t="inlineStr">
+      <c r="S20" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -2310,40 +2449,47 @@
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O21" s="5" t="inlineStr">
+      <c r="P21" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(จากรถมอเตอร์ไซค์)</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q21" s="5" t="inlineStr">
+      <c r="R21" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R21" s="5" t="inlineStr">
+      <c r="S21" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -2397,40 +2543,47 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="Q22" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q22" s="3" t="inlineStr">
+      <c r="R22" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R22" s="3" t="inlineStr">
+      <c r="S22" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -2486,40 +2639,47 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="M23" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N23" s="5" t="inlineStr">
+      <c r="O23" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O23" s="5" t="inlineStr">
+      <c r="P23" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P23" s="5" t="inlineStr">
+      <c r="Q23" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q23" s="5" t="inlineStr">
+      <c r="R23" s="5" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R23" s="5" t="inlineStr">
+      <c r="S23" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -2574,40 +2734,47 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(สุนัขข้างบ้าน รถตามถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์), กลิ่นน้ำกลิ่นน้ำจากคูน้ำตรงข้ามบ้าน)</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="R24" s="3" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R24" s="3" t="inlineStr">
+      <c r="S24" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -2660,40 +2827,47 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr">
+      <c r="M25" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M25" s="5" t="inlineStr">
+      <c r="N25" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N25" s="5" t="inlineStr">
+      <c r="O25" s="5" t="inlineStr">
         <is>
           <t>ไม่เพียงพอ</t>
         </is>
       </c>
-      <c r="O25" s="5" t="inlineStr">
+      <c r="P25" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P25" s="5" t="inlineStr">
+      <c r="Q25" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q25" s="5" t="inlineStr">
+      <c r="R25" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R25" s="5" t="inlineStr">
+      <c r="S25" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -2747,40 +2921,47 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="N26" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O26" s="3" t="inlineStr">
+      <c r="P26" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr">
+      <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q26" s="3" t="inlineStr">
+      <c r="R26" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R26" s="3" t="inlineStr">
+      <c r="S26" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -2834,40 +3015,47 @@
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr">
+      <c r="M27" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="M27" s="5" t="inlineStr">
+      <c r="N27" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N27" s="5" t="inlineStr">
+      <c r="O27" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O27" s="5" t="inlineStr">
+      <c r="P27" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, กลิ่น(มี (จากขยะ))</t>
         </is>
       </c>
-      <c r="P27" s="5" t="inlineStr">
+      <c r="Q27" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q27" s="5" t="inlineStr">
+      <c r="R27" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R27" s="5" t="inlineStr">
+      <c r="S27" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -2924,40 +3112,47 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="N28" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="O28" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr">
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(เสียง สุนัข รสตามถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
+      <c r="R28" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R28" s="3" t="inlineStr">
+      <c r="S28" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -3013,40 +3208,47 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="M29" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M29" s="5" t="inlineStr">
+      <c r="N29" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N29" s="5" t="inlineStr">
+      <c r="O29" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O29" s="5" t="inlineStr">
+      <c r="P29" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(รถสัญจร), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P29" s="5" t="inlineStr">
+      <c r="Q29" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q29" s="5" t="inlineStr">
+      <c r="R29" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R29" s="5" t="inlineStr">
+      <c r="S29" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3101,40 +3303,47 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
+      <c r="R30" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R30" s="3" t="inlineStr">
+      <c r="S30" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -3187,40 +3396,47 @@
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
+      <c r="M31" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M31" s="5" t="inlineStr">
+      <c r="N31" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N31" s="5" t="inlineStr">
+      <c r="O31" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O31" s="5" t="inlineStr">
+      <c r="P31" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(สุนัข รถบริเวณถนน), กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P31" s="5" t="inlineStr">
+      <c r="Q31" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q31" s="5" t="inlineStr">
+      <c r="R31" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R31" s="5" t="inlineStr">
+      <c r="S31" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3274,40 +3490,47 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="N32" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N32" s="3" t="inlineStr">
+      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O32" s="3" t="inlineStr">
+      <c r="P32" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q32" s="3" t="inlineStr">
+      <c r="R32" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R32" s="3" t="inlineStr">
+      <c r="S32" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3360,40 +3583,47 @@
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr">
+      <c r="M33" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M33" s="5" t="inlineStr">
+      <c r="N33" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N33" s="5" t="inlineStr">
+      <c r="O33" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O33" s="5" t="inlineStr">
+      <c r="P33" s="5" t="inlineStr">
         <is>
           <t>เสียง(เสียงรถ)</t>
         </is>
       </c>
-      <c r="P33" s="5" t="inlineStr">
+      <c r="Q33" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q33" s="5" t="inlineStr">
+      <c r="R33" s="5" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R33" s="5" t="inlineStr">
+      <c r="S33" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -3446,40 +3676,47 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="N34" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N34" s="3" t="inlineStr">
+      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O34" s="3" t="inlineStr">
+      <c r="P34" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P34" s="3" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q34" s="3" t="inlineStr">
+      <c r="R34" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R34" s="3" t="inlineStr">
+      <c r="S34" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3533,40 +3770,47 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
+      <c r="M35" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M35" s="5" t="inlineStr">
+      <c r="N35" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N35" s="5" t="inlineStr">
+      <c r="O35" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O35" s="5" t="inlineStr">
+      <c r="P35" s="5" t="inlineStr">
         <is>
           <t>เสียง(เสียงจากรถสัญจร)</t>
         </is>
       </c>
-      <c r="P35" s="5" t="inlineStr">
+      <c r="Q35" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q35" s="5" t="inlineStr">
+      <c r="R35" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R35" s="5" t="inlineStr">
+      <c r="S35" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3620,40 +3864,47 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="M36" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr">
+      <c r="N36" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N36" s="3" t="inlineStr">
+      <c r="O36" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O36" s="3" t="inlineStr">
+      <c r="P36" s="3" t="inlineStr">
         <is>
           <t>กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P36" s="3" t="inlineStr">
+      <c r="Q36" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q36" s="3" t="inlineStr">
+      <c r="R36" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R36" s="3" t="inlineStr">
+      <c r="S36" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3711,40 +3962,47 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="L37" s="5" t="inlineStr">
+      <c r="M37" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ</t>
         </is>
       </c>
-      <c r="M37" s="5" t="inlineStr">
+      <c r="N37" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N37" s="5" t="inlineStr">
+      <c r="O37" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O37" s="5" t="inlineStr">
+      <c r="P37" s="5" t="inlineStr">
         <is>
           <t>ควัน, เสียง(ติดถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P37" s="5" t="inlineStr">
+      <c r="Q37" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q37" s="5" t="inlineStr">
+      <c r="R37" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R37" s="5" t="inlineStr">
+      <c r="S37" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3798,40 +4056,47 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L38" s="3" t="inlineStr">
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr">
+      <c r="N38" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N38" s="3" t="inlineStr">
+      <c r="O38" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O38" s="3" t="inlineStr">
+      <c r="P38" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P38" s="3" t="inlineStr">
+      <c r="Q38" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q38" s="3" t="inlineStr">
+      <c r="R38" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R38" s="3" t="inlineStr">
+      <c r="S38" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3887,40 +4152,47 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="N39" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N39" s="5" t="inlineStr">
+      <c r="O39" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O39" s="5" t="inlineStr">
+      <c r="P39" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(รถสัญจรไปมา)</t>
         </is>
       </c>
-      <c r="P39" s="5" t="inlineStr">
+      <c r="Q39" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q39" s="5" t="inlineStr">
+      <c r="R39" s="5" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R39" s="5" t="inlineStr">
+      <c r="S39" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -3975,40 +4247,47 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L40" s="3" t="inlineStr">
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M40" s="3" t="inlineStr">
+      <c r="N40" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N40" s="3" t="inlineStr">
+      <c r="O40" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O40" s="3" t="inlineStr">
+      <c r="P40" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P40" s="3" t="inlineStr">
+      <c r="Q40" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q40" s="3" t="inlineStr">
+      <c r="R40" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R40" s="3" t="inlineStr">
+      <c r="S40" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -4063,40 +4342,47 @@
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L41" s="5" t="inlineStr">
+      <c r="M41" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M41" s="5" t="inlineStr">
+      <c r="N41" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N41" s="5" t="inlineStr">
+      <c r="O41" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O41" s="5" t="inlineStr">
+      <c r="P41" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(เสียงสุนัขเห่า), กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P41" s="5" t="inlineStr">
+      <c r="Q41" s="5" t="inlineStr">
         <is>
           <t>เผา, อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q41" s="5" t="inlineStr">
+      <c r="R41" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R41" s="5" t="inlineStr">
+      <c r="S41" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -4150,40 +4436,47 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L42" s="3" t="inlineStr">
+      <c r="M42" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M42" s="3" t="inlineStr">
+      <c r="N42" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N42" s="3" t="inlineStr">
+      <c r="O42" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O42" s="3" t="inlineStr">
+      <c r="P42" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P42" s="3" t="inlineStr">
+      <c r="Q42" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q42" s="3" t="inlineStr">
+      <c r="R42" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R42" s="3" t="inlineStr">
+      <c r="S42" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -4236,40 +4529,47 @@
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L43" s="5" t="inlineStr">
+      <c r="M43" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M43" s="5" t="inlineStr">
+      <c r="N43" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N43" s="5" t="inlineStr">
+      <c r="O43" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O43" s="5" t="inlineStr">
+      <c r="P43" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(ติดถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P43" s="5" t="inlineStr">
+      <c r="Q43" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q43" s="5" t="inlineStr">
+      <c r="R43" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R43" s="5" t="inlineStr">
+      <c r="S43" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -4326,40 +4626,47 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L44" s="3" t="inlineStr">
+      <c r="M44" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M44" s="3" t="inlineStr">
+      <c r="N44" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N44" s="3" t="inlineStr">
+      <c r="O44" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O44" s="3" t="inlineStr">
+      <c r="P44" s="3" t="inlineStr">
         <is>
           <t>เสียง(เสียงรถสัญจร)</t>
         </is>
       </c>
-      <c r="P44" s="3" t="inlineStr">
+      <c r="Q44" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q44" s="3" t="inlineStr">
+      <c r="R44" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R44" s="3" t="inlineStr">
+      <c r="S44" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -4412,40 +4719,47 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L45" s="5" t="inlineStr">
+      <c r="M45" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M45" s="5" t="inlineStr">
+      <c r="N45" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N45" s="5" t="inlineStr">
+      <c r="O45" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O45" s="5" t="inlineStr">
+      <c r="P45" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(ติดถนน), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P45" s="5" t="inlineStr">
+      <c r="Q45" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q45" s="5" t="inlineStr">
+      <c r="R45" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R45" s="5" t="inlineStr">
+      <c r="S45" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -4501,40 +4815,47 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L46" s="3" t="inlineStr">
+      <c r="M46" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M46" s="3" t="inlineStr">
+      <c r="N46" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N46" s="3" t="inlineStr">
+      <c r="O46" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O46" s="3" t="inlineStr">
+      <c r="P46" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P46" s="3" t="inlineStr">
+      <c r="Q46" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q46" s="3" t="inlineStr">
+      <c r="R46" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R46" s="3" t="inlineStr">
+      <c r="S46" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -4589,40 +4910,47 @@
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L47" s="5" t="inlineStr">
+      <c r="M47" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M47" s="5" t="inlineStr">
+      <c r="N47" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N47" s="5" t="inlineStr">
+      <c r="O47" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O47" s="5" t="inlineStr">
+      <c r="P47" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(เสียงรถ)</t>
         </is>
       </c>
-      <c r="P47" s="5" t="inlineStr">
+      <c r="Q47" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q47" s="5" t="inlineStr">
+      <c r="R47" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R47" s="5" t="inlineStr">
+      <c r="S47" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -4676,40 +5004,47 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L48" s="3" t="inlineStr">
+      <c r="M48" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M48" s="3" t="inlineStr">
+      <c r="N48" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N48" s="3" t="inlineStr">
+      <c r="O48" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O48" s="3" t="inlineStr">
+      <c r="P48" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(รถสัญจรไปมา)</t>
         </is>
       </c>
-      <c r="P48" s="3" t="inlineStr">
+      <c r="Q48" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q48" s="3" t="inlineStr">
+      <c r="R48" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R48" s="3" t="inlineStr">
+      <c r="S48" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -4765,40 +5100,47 @@
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L49" s="5" t="inlineStr">
+      <c r="M49" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M49" s="5" t="inlineStr">
+      <c r="N49" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N49" s="5" t="inlineStr">
+      <c r="O49" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O49" s="5" t="inlineStr">
+      <c r="P49" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P49" s="5" t="inlineStr">
+      <c r="Q49" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q49" s="5" t="inlineStr">
+      <c r="R49" s="5" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R49" s="5" t="inlineStr">
+      <c r="S49" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -4852,40 +5194,47 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L50" s="3" t="inlineStr">
+      <c r="M50" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M50" s="3" t="inlineStr">
+      <c r="N50" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N50" s="3" t="inlineStr">
+      <c r="O50" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O50" s="3" t="inlineStr">
+      <c r="P50" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, เสียง(เสียงรถสัญจร)</t>
         </is>
       </c>
-      <c r="P50" s="3" t="inlineStr">
+      <c r="Q50" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q50" s="3" t="inlineStr">
+      <c r="R50" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R50" s="3" t="inlineStr">
+      <c r="S50" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -4940,40 +5289,47 @@
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L51" s="5" t="inlineStr">
+      <c r="M51" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M51" s="5" t="inlineStr">
+      <c r="N51" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N51" s="5" t="inlineStr">
+      <c r="O51" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O51" s="5" t="inlineStr">
+      <c r="P51" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P51" s="5" t="inlineStr">
+      <c r="Q51" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q51" s="5" t="inlineStr">
+      <c r="R51" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R51" s="5" t="inlineStr">
+      <c r="S51" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -5029,40 +5385,47 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L52" s="3" t="inlineStr">
+      <c r="M52" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M52" s="3" t="inlineStr">
+      <c r="N52" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N52" s="3" t="inlineStr">
+      <c r="O52" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O52" s="3" t="inlineStr">
+      <c r="P52" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P52" s="3" t="inlineStr">
+      <c r="Q52" s="3" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q52" s="3" t="inlineStr">
+      <c r="R52" s="3" t="inlineStr">
         <is>
           <t>บ่อน้ำทิ้ง</t>
         </is>
       </c>
-      <c r="R52" s="3" t="inlineStr">
+      <c r="S52" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -5120,40 +5483,47 @@
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L53" s="5" t="inlineStr">
+      <c r="M53" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M53" s="5" t="inlineStr">
+      <c r="N53" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N53" s="5" t="inlineStr">
+      <c r="O53" s="5" t="inlineStr">
         <is>
           <t>ไม่เพียงพอ</t>
         </is>
       </c>
-      <c r="O53" s="5" t="inlineStr">
+      <c r="P53" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(รถส่งของโรงงาน), กลิ่น(มี (จากขยะ))</t>
         </is>
       </c>
-      <c r="P53" s="5" t="inlineStr">
+      <c r="Q53" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q53" s="5" t="inlineStr">
+      <c r="R53" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R53" s="5" t="inlineStr">
+      <c r="S53" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -5207,40 +5577,47 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L54" s="3" t="inlineStr">
+      <c r="M54" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M54" s="3" t="inlineStr">
+      <c r="N54" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N54" s="3" t="inlineStr">
+      <c r="O54" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O54" s="3" t="inlineStr">
+      <c r="P54" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P54" s="3" t="inlineStr">
+      <c r="Q54" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q54" s="3" t="inlineStr">
+      <c r="R54" s="3" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R54" s="3" t="inlineStr">
+      <c r="S54" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -5297,40 +5674,47 @@
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L55" s="5" t="inlineStr">
+      <c r="M55" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M55" s="5" t="inlineStr">
+      <c r="N55" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N55" s="5" t="inlineStr">
+      <c r="O55" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O55" s="5" t="inlineStr">
+      <c r="P55" s="5" t="inlineStr">
         <is>
           <t>ควัน, เสียง(รถเครื่อง)</t>
         </is>
       </c>
-      <c r="P55" s="5" t="inlineStr">
+      <c r="Q55" s="5" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q55" s="5" t="inlineStr">
+      <c r="R55" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R55" s="5" t="inlineStr">
+      <c r="S55" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -5385,40 +5769,47 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L56" s="3" t="inlineStr">
+      <c r="M56" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M56" s="3" t="inlineStr">
+      <c r="N56" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N56" s="3" t="inlineStr">
+      <c r="O56" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O56" s="3" t="inlineStr">
+      <c r="P56" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P56" s="3" t="inlineStr">
+      <c r="Q56" s="3" t="inlineStr">
         <is>
           <t>ฝากลูกไปทิ้งที่ทางด่วน</t>
         </is>
       </c>
-      <c r="Q56" s="3" t="inlineStr">
+      <c r="R56" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R56" s="3" t="inlineStr">
+      <c r="S56" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -5475,40 +5866,47 @@
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L57" s="5" t="inlineStr">
+      <c r="M57" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M57" s="5" t="inlineStr">
+      <c r="N57" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N57" s="5" t="inlineStr">
+      <c r="O57" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O57" s="5" t="inlineStr">
+      <c r="P57" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(เสียงรถ), กลิ่น(กลิ่นสี)</t>
         </is>
       </c>
-      <c r="P57" s="5" t="inlineStr">
+      <c r="Q57" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q57" s="5" t="inlineStr">
+      <c r="R57" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R57" s="5" t="inlineStr">
+      <c r="S57" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -5562,40 +5960,47 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L58" s="3" t="inlineStr">
+      <c r="M58" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M58" s="3" t="inlineStr">
+      <c r="N58" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N58" s="3" t="inlineStr">
+      <c r="O58" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O58" s="3" t="inlineStr">
+      <c r="P58" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(ติดถนน)</t>
         </is>
       </c>
-      <c r="P58" s="3" t="inlineStr">
+      <c r="Q58" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q58" s="3" t="inlineStr">
+      <c r="R58" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R58" s="3" t="inlineStr">
+      <c r="S58" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -5648,40 +6053,47 @@
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L59" s="5" t="inlineStr">
+      <c r="M59" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M59" s="5" t="inlineStr">
+      <c r="N59" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N59" s="5" t="inlineStr">
+      <c r="O59" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O59" s="5" t="inlineStr">
+      <c r="P59" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P59" s="5" t="inlineStr">
+      <c r="Q59" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q59" s="5" t="inlineStr">
+      <c r="R59" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R59" s="5" t="inlineStr">
+      <c r="S59" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -5735,40 +6147,47 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L60" s="3" t="inlineStr">
+      <c r="M60" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M60" s="3" t="inlineStr">
+      <c r="N60" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N60" s="3" t="inlineStr">
+      <c r="O60" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O60" s="3" t="inlineStr">
+      <c r="P60" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P60" s="3" t="inlineStr">
+      <c r="Q60" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q60" s="3" t="inlineStr">
+      <c r="R60" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R60" s="3" t="inlineStr">
+      <c r="S60" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -5823,40 +6242,47 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L61" s="5" t="inlineStr">
+      <c r="M61" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M61" s="5" t="inlineStr">
+      <c r="N61" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N61" s="5" t="inlineStr">
+      <c r="O61" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O61" s="5" t="inlineStr">
+      <c r="P61" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P61" s="5" t="inlineStr">
+      <c r="Q61" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q61" s="5" t="inlineStr">
+      <c r="R61" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R61" s="5" t="inlineStr">
+      <c r="S61" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -5910,40 +6336,47 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ทราบ
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L62" s="3" t="inlineStr">
+      <c r="M62" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M62" s="3" t="inlineStr">
+      <c r="N62" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N62" s="3" t="inlineStr">
+      <c r="O62" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O62" s="3" t="inlineStr">
+      <c r="P62" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P62" s="3" t="inlineStr">
+      <c r="Q62" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q62" s="3" t="inlineStr">
+      <c r="R62" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R62" s="3" t="inlineStr">
+      <c r="S62" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -5998,40 +6431,47 @@
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L63" s="5" t="inlineStr">
+      <c r="M63" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M63" s="5" t="inlineStr">
+      <c r="N63" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N63" s="5" t="inlineStr">
+      <c r="O63" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O63" s="5" t="inlineStr">
+      <c r="P63" s="5" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P63" s="5" t="inlineStr">
+      <c r="Q63" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q63" s="5" t="inlineStr">
+      <c r="R63" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R63" s="5" t="inlineStr">
+      <c r="S63" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -6084,40 +6524,47 @@
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L64" s="3" t="inlineStr">
+      <c r="M64" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M64" s="3" t="inlineStr">
+      <c r="N64" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N64" s="3" t="inlineStr">
+      <c r="O64" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O64" s="3" t="inlineStr">
+      <c r="P64" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, เสียง(สุนัข รถ), กลิ่น(มี (จากขยะ), มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P64" s="3" t="inlineStr">
+      <c r="Q64" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q64" s="3" t="inlineStr">
+      <c r="R64" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R64" s="3" t="inlineStr">
+      <c r="S64" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -6173,40 +6620,47 @@
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L65" s="5" t="inlineStr">
+      <c r="M65" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M65" s="5" t="inlineStr">
+      <c r="N65" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N65" s="5" t="inlineStr">
+      <c r="O65" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O65" s="5" t="inlineStr">
+      <c r="P65" s="5" t="inlineStr">
         <is>
           <t>เสียง(รถสัญจร)</t>
         </is>
       </c>
-      <c r="P65" s="5" t="inlineStr">
+      <c r="Q65" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q65" s="5" t="inlineStr">
+      <c r="R65" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R65" s="5" t="inlineStr">
+      <c r="S65" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -6261,40 +6715,47 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ไม่ตามเกณฑ์
+น้ำตาล: ไม่ตามเกณฑ์
+น้ำมัน: ไม่ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L66" s="3" t="inlineStr">
+      <c r="M66" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M66" s="3" t="inlineStr">
+      <c r="N66" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทไม่สะดวก</t>
         </is>
       </c>
-      <c r="N66" s="3" t="inlineStr">
+      <c r="O66" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O66" s="3" t="inlineStr">
+      <c r="P66" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง</t>
         </is>
       </c>
-      <c r="P66" s="3" t="inlineStr">
+      <c r="Q66" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q66" s="3" t="inlineStr">
+      <c r="R66" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R66" s="3" t="inlineStr">
+      <c r="S66" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -6350,40 +6811,47 @@
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L67" s="5" t="inlineStr">
+      <c r="M67" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M67" s="5" t="inlineStr">
+      <c r="N67" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N67" s="5" t="inlineStr">
+      <c r="O67" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O67" s="5" t="inlineStr">
+      <c r="P67" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, ควัน, กลิ่น(บ่อปลา ปลาตาย)</t>
         </is>
       </c>
-      <c r="P67" s="5" t="inlineStr">
+      <c r="Q67" s="5" t="inlineStr">
         <is>
           <t>เผา, อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q67" s="5" t="inlineStr">
+      <c r="R67" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R67" s="5" t="inlineStr">
+      <c r="S67" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -6436,40 +6904,47 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L68" s="3" t="inlineStr">
+      <c r="M68" s="3" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M68" s="3" t="inlineStr">
+      <c r="N68" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N68" s="3" t="inlineStr">
+      <c r="O68" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O68" s="3" t="inlineStr">
+      <c r="P68" s="3" t="inlineStr">
         <is>
           <t>ไม่มีปัญหา</t>
         </is>
       </c>
-      <c r="P68" s="3" t="inlineStr">
+      <c r="Q68" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q68" s="3" t="inlineStr">
+      <c r="R68" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R68" s="3" t="inlineStr">
+      <c r="S68" s="3" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>
@@ -6527,40 +7002,47 @@
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L69" s="5" t="inlineStr">
+      <c r="M69" s="5" t="inlineStr">
         <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="M69" s="5" t="inlineStr">
+      <c r="N69" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N69" s="5" t="inlineStr">
+      <c r="O69" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O69" s="5" t="inlineStr">
+      <c r="P69" s="5" t="inlineStr">
         <is>
           <t>ควัน, เสียง(รถเครื่องยนต์)</t>
         </is>
       </c>
-      <c r="P69" s="5" t="inlineStr">
+      <c r="Q69" s="5" t="inlineStr">
         <is>
           <t>เผา</t>
         </is>
       </c>
-      <c r="Q69" s="5" t="inlineStr">
+      <c r="R69" s="5" t="inlineStr">
         <is>
           <t>ร่องระบายน้ำของหมู่บ้าน</t>
         </is>
       </c>
-      <c r="R69" s="5" t="inlineStr">
+      <c r="S69" s="5" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -6618,40 +7100,47 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
           <t>เป็นระเบียบ, สะอาด</t>
         </is>
       </c>
-      <c r="L70" s="3" t="inlineStr">
+      <c r="M70" s="3" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M70" s="3" t="inlineStr">
+      <c r="N70" s="3" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N70" s="3" t="inlineStr">
+      <c r="O70" s="3" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O70" s="3" t="inlineStr">
+      <c r="P70" s="3" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P70" s="3" t="inlineStr">
+      <c r="Q70" s="3" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q70" s="3" t="inlineStr">
+      <c r="R70" s="3" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R70" s="3" t="inlineStr">
+      <c r="S70" s="3" t="inlineStr">
         <is>
           <t>เลี้ยง</t>
         </is>
@@ -6704,40 +7193,47 @@
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
+          <t>โซเดียม: ตามเกณฑ์
+น้ำตาล: ตามเกณฑ์
+น้ำมัน: ตามเกณฑ์</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="L71" s="5" t="inlineStr">
+      <c r="M71" s="5" t="inlineStr">
         <is>
           <t>ไม่เป็นระเบียบ, ไม่สะอาด</t>
         </is>
       </c>
-      <c r="M71" s="5" t="inlineStr">
+      <c r="N71" s="5" t="inlineStr">
         <is>
           <t>ถ่ายเทสะดวก</t>
         </is>
       </c>
-      <c r="N71" s="5" t="inlineStr">
+      <c r="O71" s="5" t="inlineStr">
         <is>
           <t>เพียงพอ</t>
         </is>
       </c>
-      <c r="O71" s="5" t="inlineStr">
+      <c r="P71" s="5" t="inlineStr">
         <is>
           <t>ฝุ่นละออง, กลิ่น(มี (จากมูลสัตว์))</t>
         </is>
       </c>
-      <c r="P71" s="5" t="inlineStr">
+      <c r="Q71" s="5" t="inlineStr">
         <is>
           <t>อบต./เทศบาลมาเก็บ</t>
         </is>
       </c>
-      <c r="Q71" s="5" t="inlineStr">
+      <c r="R71" s="5" t="inlineStr">
         <is>
           <t>ทิ้งลงบนพื้นดิน</t>
         </is>
       </c>
-      <c r="R71" s="5" t="inlineStr">
+      <c r="S71" s="5" t="inlineStr">
         <is>
           <t>ไม่เลี้ยง</t>
         </is>

</xml_diff>

<commit_message>
Update exact age values across all 204 members in Excel and Dashboard
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>รายชื่อสมาชิกทั้งหมด</t>
+          <t>รายชื่อสมาชิกทั้งหมด (อายุจริง)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -623,15 +623,15 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1. นางสาวเพ็ญนภา บุญเสริม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางราวี เวียงสมุทร (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายถาวร เวียงสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-4. นางภิรมณ์พร บุญจันที (หญิง, 45–59 ปี, ครูผู้ช่วย)
-5. นางสาวกัญญารัตน์ อัมไพ (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางสาวเพ็ญนภา บุญเสริม (หญิง, อายุ 56 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางราวี เวียงสมุทร (หญิง, อายุ 75 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายถาวร เวียงสมุทร (ชาย, อายุ 87 ปี, ไม่ได้ประกอบอาชีพ)
+4. นางภิรมณ์พร บุญจันที (หญิง, อายุ 50 ปี, ครูผู้ช่วย)
+5. นางสาวกัญญารัตน์ อัมไพ (หญิง, อายุ 17 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
@@ -720,9 +720,9 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>1. นฤมล บุญรอด (หญิง, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
-2. อำนวย นามนาค (ชาย, 45–59 ปี, พนักงานบริษัท)
-3. สุวิลักขณ์ นามนาค (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นฤมล บุญรอด (หญิง, อายุ 50 ปี, ไม่ได้ประกอบอาชีพ)
+2. อำนวย นามนาค (ชาย, อายุ 52 ปี, พนักงานบริษัท)
+3. สุวิลักขณ์ นามนาค (ชาย, อายุ 11 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G3" s="4" t="n">
@@ -815,10 +815,10 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1. นายทองคำ เลิศพาณุมาศ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสุมาลี พวงโคสน (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายประสิทธิ์ เลิศพาณุมาศ (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)
-4. ด.ช.ปนชัย เลิศพาณุมาศ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นายทองคำ เลิศพาณุมาศ (ชาย, อายุ 66 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางสุมาลี พวงโคสน (หญิง, อายุ 60 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายประสิทธิ์ เลิศพาณุมาศ (ชาย, อายุ 35 ปี, ไม่ได้ประกอบอาชีพ)
+4. ด.ช.ปนชัย เลิศพาณุมาศ (ชาย, อายุ 14 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
@@ -911,9 +911,9 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวบุษรา เพชรรัตน์ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นางทองอยู่ เพชรรัตน์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายอารมณ์ เพชรรัตน์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวบุษรา เพชรรัตน์ (หญิง, อายุ 56 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นางทองอยู่ เพชรรัตน์ (ชาย, อายุ 75 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายอารมณ์ เพชรรัตน์ (ชาย, อายุ 74 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G5" s="4" t="n">
@@ -1006,8 +1006,8 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1. เล็ก สมบัติเปี่ยม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. เยียน สมบัติเปี่ยม (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. เล็ก สมบัติเปี่ยม (หญิง, อายุ 93 ปี, ไม่ได้ประกอบอาชีพ)
+2. เยียน สมบัติเปี่ยม (ชาย, อายุ 87 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
@@ -1100,10 +1100,10 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>1. นายนุกุล อยู่สุข (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นางนงนุช อยู่สุข (หญิง, 45–59 ปี, เกษตรกรรม)
-3. นายธนดล อยู่สุข (ชาย, 25–44 ปี, เกษตรกรรม)
-4. นางวรัญธร อยู่สุข (หญิง, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายนุกุล อยู่สุข (ชาย, อายุ 60 ปี, เกษตรกรรม)
+2. นางนงนุช อยู่สุข (หญิง, อายุ 59 ปี, เกษตรกรรม)
+3. นายธนดล อยู่สุข (ชาย, อายุ 37 ปี, เกษตรกรรม)
+4. นางวรัญธร อยู่สุข (หญิง, อายุ 33 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G7" s="4" t="n">
@@ -1196,9 +1196,9 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>1. นาง ฉลวย รัตนะ (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายอำนาจนายอำนาจ พรมทัศน์ (ชาย, 25–44 ปี, รับจ้าง)
-3. เด็กหญิงธิติมา สาธุจรัญ (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นาง ฉลวย รัตนะ (หญิง, อายุ 63 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายอำนาจนายอำนาจ พรมทัศน์ (ชาย, อายุ 30 ปี, รับจ้าง)
+3. เด็กหญิงธิติมา สาธุจรัญ (หญิง, อายุ 15 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
@@ -1291,9 +1291,9 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>1. นางสุชิน  ชีวงค์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นายอนุชา เพชรรัตน์ (ชาย, 45–59 ปี, รับจ้าง)
-3. นายภควัฒน์ หนองใหญ่ (ชาย, 15–24 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสุชิน  ชีวงค์ (หญิง, อายุ 69 ปี, ไม่ได้ประกอบอาชีพ)
+2. นายอนุชา เพชรรัตน์ (ชาย, อายุ 48 ปี, รับจ้าง)
+3. นายภควัฒน์ หนองใหญ่ (ชาย, อายุ 18 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
@@ -1386,10 +1386,10 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>1. เพลินจิต ทองเจือ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. สมนึก ทองเจือ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. ภัควัตร ทองเจือ (ชาย, 25–44 ปี, รับจ้าง)
-4. สมคิด ทองเจือ (หญิง, 60 ปีขึ้นไป, รับจ้าง)</t>
+          <t>1. เพลินจิต ทองเจือ (หญิง, อายุ 77 ปี, ไม่ได้ประกอบอาชีพ)
+2. สมนึก ทองเจือ (ชาย, อายุ 73 ปี, ไม่ได้ประกอบอาชีพ)
+3. ภัควัตร ทองเจือ (ชาย, อายุ 35 ปี, รับจ้าง)
+4. สมคิด ทองเจือ (หญิง, อายุ 79 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวสุชิรา รื่นเริง (หญิง, 45–59 ปี, ช่วยเลี้ยงหลาน)</t>
+          <t>1. นางสาวสุชิรา รื่นเริง (หญิง, อายุ 49 ปี, ช่วยเลี้ยงหลาน)</t>
         </is>
       </c>
       <c r="G11" s="4" t="n">
@@ -1575,11 +1575,11 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>1. นายถวัลย์ คำประสิทธิ์ (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางไพรัตน์ คำประสิทธิ์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายกิตติพงศ์ คำประสิทธิ์ (ชาย, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. นายพงศธร คำประสิทธิ์ (ชาย, 45–59 ปี, รับจ้าง)
-5. นางกมลรัตน์ คำประสิทธิ์ (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
+          <t>1. นายถวัลย์ คำประสิทธิ์ (ชาย, อายุ 73 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางไพรัตน์ คำประสิทธิ์ (หญิง, อายุ 67 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายกิตติพงศ์ คำประสิทธิ์ (ชาย, อายุ 47 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. นายพงศธร คำประสิทธิ์ (ชาย, อายุ 46 ปี, รับจ้าง)
+5. นางกมลรัตน์ คำประสิทธิ์ (หญิง, อายุ 45 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
@@ -1672,8 +1672,8 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>1. บุปผา ทิพย์กานนท์ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. เฉลิมพล ทิพย์กานนท์ (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. บุปผา ทิพย์กานนท์ (หญิง, อายุ 55 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. เฉลิมพล ทิพย์กานนท์ (ชาย, อายุ 58 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G13" s="4" t="n">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>1. นางสวง ช่วยรักษา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสวง ช่วยรักษา (หญิง, อายุ 71 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
@@ -1859,9 +1859,9 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>1. นางสำนางสำรวย เมตตา (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. นานปนวรรณ สาแหลกทอง (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)
-3. นายจตุรงค์ เมตตา (ชาย, 25–44 ปี, รปภ.)</t>
+          <t>1. นางสำนางสำรวย เมตตา (หญิง, อายุ 78 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นานปนวรรณ สาแหลกทอง (ชาย, อายุ 26 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายจตุรงค์ เมตตา (ชาย, อายุ 40 ปี, รปภ.)</t>
         </is>
       </c>
       <c r="G15" s="4" t="n">
@@ -1950,10 +1950,10 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>1. นางจุฑารัตน์ บุญคำ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายสมศักดิ์ ฉั่วยู่เน้ย (ชาย, 45–59 ปี, รับจ้าง)
-3. นายธนดล ฉั่วยู่เน้ย (ชาย, 25–44 ปี, รับจ้าง)
-4. นางสาวอินทิรา ฉั่วยู่เน้ย (หญิง, 15–24 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางจุฑารัตน์ บุญคำ (หญิง, อายุ 49 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายสมศักดิ์ ฉั่วยู่เน้ย (ชาย, อายุ 49 ปี, รับจ้าง)
+3. นายธนดล ฉั่วยู่เน้ย (ชาย, อายุ 26 ปี, รับจ้าง)
+4. นางสาวอินทิรา ฉั่วยู่เน้ย (หญิง, อายุ 24 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
@@ -2046,14 +2046,14 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>1. ประเทือง พูลศิริ (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. เฉลิม พูลศิริ (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. เอมอร (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. บรรพต ทองอินทร์ (ชาย, 60 ปีขึ้นไป, รับราชการ/รัฐวิสาหกิจ)</t>
+          <t>1. ประเทือง พูลศิริ (หญิง, อายุ 78 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. เฉลิม พูลศิริ (ชาย, อายุ 84 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. เอมอร (หญิง, อายุ 55 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. บรรพต ทองอินทร์ (ชาย, อายุ 57 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>1. นางอำพร คงผ่องแผ้ว (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. นางอำพร คงผ่องแผ้ว (หญิง, อายุ 73 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
@@ -2235,11 +2235,11 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>1. นางบุญเรือง พรมทัศน์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)
-2. นางสาวมยุรีย์ พรมทัศน์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)
-3. นางสาวธนพัฒน์ บุญช่วย (หญิง, 25–44 ปี, พนักงานบริษัท)
-4. นายธนวัฒน์ บุญช่วย (ชาย, 25–44 ปี, รับจ้าง)
-5. เด็กชายชัชธนนฌ์ วโรธรวัช (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางบุญเรือง พรมทัศน์ (หญิง, อายุ 71 ปี, รับจ้าง)
+2. นางสาวมยุรีย์ พรมทัศน์ (หญิง, อายุ 62 ปี, รับจ้าง)
+3. นางสาวธนพัฒน์ บุญช่วย (หญิง, อายุ 34 ปี, พนักงานบริษัท)
+4. นายธนวัฒน์ บุญช่วย (ชาย, อายุ 33 ปี, รับจ้าง)
+5. เด็กชายชัชธนนฌ์ วโรธรวัช (ชาย, อายุ 4 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G19" s="4" t="n">
@@ -2332,8 +2332,8 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>1. สมหมาย หนูเกต (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายศุทินันท์ หนูเกต (ชาย, 25–44 ปี, รับจ้าง)</t>
+          <t>1. สมหมาย หนูเกต (ชาย, อายุ 65 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายศุทินันท์ หนูเกต (ชาย, อายุ 29 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวมาลัย องคศิลป์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวมาลัย องคศิลป์ (หญิง, อายุ 80 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G21" s="4" t="n">
@@ -2519,8 +2519,8 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>1. นายบรรจง บุญรอด (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสาวพรพิมล พูนศิริ (หญิง, 25–44 ปี, พยาบาล)</t>
+          <t>1. นายบรรจง บุญรอด (ชาย, อายุ 80 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางสาวพรพิมล พูนศิริ (หญิง, อายุ 35 ปี, พยาบาล)</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
@@ -2613,10 +2613,10 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>1. สังวาลย์ สุขสว่าง (หญิง, 60 ปีขึ้นไป, รับจ้าง)
-2. สมหวัง สุขสว่าง (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. ภาคภูมิ สุขสว่าง (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-4. พีรพล สุขสว่าง (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. สังวาลย์ สุขสว่าง (หญิง, อายุ 61 ปี, รับจ้าง)
+2. สมหวัง สุขสว่าง (ชาย, อายุ 42 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. ภาคภูมิ สุขสว่าง (ชาย, อายุ 11 ปี, นักเรียน/นักศึกษา)
+4. พีรพล สุขสว่าง (ชาย, อายุ 9 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
@@ -2709,9 +2709,9 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>1. นางสาวสาวินีย์ สีกาสี (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายอิงอร โม่ไหม (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. เด็กหญิงสรินพร โม่ไหม (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางสาวสาวินีย์ สีกาสี (หญิง, อายุ 45 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายอิงอร โม่ไหม (ชาย, อายุ 52 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. เด็กหญิงสรินพร โม่ไหม (หญิง, อายุ 7 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>1. นางประยงค์ พรหมทัศน์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางประยงค์ พรหมทัศน์ (หญิง, อายุ 71 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G25" s="4" t="n">
@@ -2897,8 +2897,8 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>1. นายประวิทย์ บุญช่วย (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางบุญยืน บุญช่วย (หญิง, 60 ปีขึ้นไป, อสม)</t>
+          <t>1. นายประวิทย์ บุญช่วย (ชาย, อายุ 71 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางบุญยืน บุญช่วย (หญิง, อายุ 69 ปี, อสม)</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
@@ -2991,8 +2991,8 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>1. นายสมคิด เวียงสมุทร (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นางส้มเกลี้ยง เวียงสมุทร (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายสมคิด เวียงสมุทร (ชาย, อายุ 65 ปี, เกษตรกรรม)
+2. นางส้มเกลี้ยง เวียงสมุทร (หญิง, อายุ 89 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G27" s="4" t="n">
@@ -3085,11 +3085,11 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>1. นภา สวนรักษา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. คำรณค์ สวนรักษา (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. นพดล สวนรักษา (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-4. พงษกรณ์ สวนรักษา (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)
-5. ภรกรณ์ สวนรักษา (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นภา สวนรักษา (หญิง, อายุ 77 ปี, ไม่ได้ประกอบอาชีพ)
+2. คำรณค์ สวนรักษา (ชาย, อายุ 48 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. นพดล สวนรักษา (ชาย, อายุ 43 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+4. พงษกรณ์ สวนรักษา (ชาย, อายุ 17 ปี, นักเรียน/นักศึกษา)
+5. ภรกรณ์ สวนรักษา (ชาย, อายุ 17 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
@@ -3182,10 +3182,10 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>1. นางอ้อย อยู่สุข (หญิง, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นายรุ่ง ปามา (ชาย, 60 ปีขึ้นไป, รับจ้าง)
-3. นายธีรภัทร พรหมพัฒน์ (ชาย, 15–24 ปี, รับจ้าง)
-4. นางสาววัชนี พรหมพัฒน์ (หญิง, 15–24 ปี, รับจ้าง)</t>
+          <t>1. นางอ้อย อยู่สุข (หญิง, อายุ 61 ปี, เกษตรกรรม)
+2. นายรุ่ง ปามา (ชาย, อายุ 66 ปี, รับจ้าง)
+3. นายธีรภัทร พรหมพัฒน์ (ชาย, อายุ 23 ปี, รับจ้าง)
+4. นางสาววัชนี พรหมพัฒน์ (หญิง, อายุ 23 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G29" s="4" t="n">
@@ -3278,13 +3278,13 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>1. ไพทูรย์ โชคชัยฤทธิ์ (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ปทุม เมฆจั่น (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. พลอยรัตน์ โชคชัยฤทธิ์ (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. ไพทูรย์ โชคชัยฤทธิ์ (ชาย, อายุ 59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. ปทุม เมฆจั่น (หญิง, อายุ 48 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. พลอยรัตน์ โชคชัยฤทธิ์ (หญิง, อายุ 10 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวอรนุช คุ้มทรัพย์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวอรนุช คุ้มทรัพย์ (หญิง, อายุ 75 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G31" s="4" t="n">
@@ -3466,8 +3466,8 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>1. นายประเสริฐ เกศมาลา (ชาย, 60 ปีขึ้นไป, ได้รายได้จากลูกชาย)
-2. นางนางใจ เกศมาลา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายประเสริฐ เกศมาลา (ชาย, อายุ 75 ปี, ได้รายได้จากลูกชาย)
+2. นางนางใจ เกศมาลา (หญิง, อายุ 65 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>1. นาวสำรวย คงผงแผ้ว (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นาวสำรวย คงผงแผ้ว (หญิง, อายุ 83 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G33" s="4" t="n">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>1. ภัทรทาดา ทองคำ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ภัทรทาดา ทองคำ (หญิง, อายุ 42 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
@@ -3746,8 +3746,8 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>1. นายมนตรี มนต์คจรเดชา (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นางมาลี มนต์คจรเดชา (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายมนตรี มนต์คจรเดชา (ชาย, อายุ 64 ปี, เกษตรกรรม)
+2. นางมาลี มนต์คจรเดชา (หญิง, อายุ 89 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G35" s="4" t="n">
@@ -3840,8 +3840,8 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>1. นายโฉม ชัยศรีเกษมพันธุ์ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นางลำเพย ชัยศรีเกษมพันธุ์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)</t>
+          <t>1. นายโฉม ชัยศรีเกษมพันธุ์ (ชาย, อายุ 70 ปี, เกษตรกรรม)
+2. นางลำเพย ชัยศรีเกษมพันธุ์ (หญิง, อายุ 65 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>1. ลภัสลดา ผู้ทัด (หญิง, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
-2. สาลี่ บุญรอด (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. อภิวัฒน์ ผู้ทัด (ชาย, 15–24 ปี, รับจ้าง)
-4. รัตนาภร อเนก (หญิง, 15–24 ปี, รับจ้าง)
-5. ภิรมย์ ผู้ทัด (ชาย, 45–59 ปี, รับจ้าง)
-6. พราวณิรินทร์ ผู้ทัด (หญิง, ต่ำกว่า 15 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ลภัสลดา ผู้ทัด (หญิง, อายุ 48 ปี, ไม่ได้ประกอบอาชีพ)
+2. สาลี่ บุญรอด (หญิง, อายุ 69 ปี, ไม่ได้ประกอบอาชีพ)
+3. อภิวัฒน์ ผู้ทัด (ชาย, อายุ 21 ปี, รับจ้าง)
+4. รัตนาภร อเนก (หญิง, อายุ 22 ปี, รับจ้าง)
+5. ภิรมย์ ผู้ทัด (ชาย, อายุ 50 ปี, รับจ้าง)
+6. พราวณิรินทร์ ผู้ทัด (หญิง, อายุ 1 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G37" s="4" t="n">
@@ -4032,8 +4032,8 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>1. สนอง ทองคำ (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. สุขสันต์ เลิศรัตน์ (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. สนอง ทองคำ (ชาย, อายุ 68 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. สุขสันต์ เลิศรัตน์ (ชาย, อายุ 48 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
@@ -4126,10 +4126,10 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>1. ธัญพร บุญรอด (หญิง, 45–59 ปี, รายได้จากสามี)
-2. ณัฐพล อรวีรนนท์ (ชาย, 45–59 ปี, ขับแท็กซี่)
-3. อุทัย บุญรอด (ชาย, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
-4. สุดารัตน์ บุญรอด (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ธัญพร บุญรอด (หญิง, อายุ 57 ปี, รายได้จากสามี)
+2. ณัฐพล อรวีรนนท์ (ชาย, อายุ 58 ปี, ขับแท็กซี่)
+3. อุทัย บุญรอด (ชาย, อายุ 54 ปี, ไม่ได้ประกอบอาชีพ)
+4. สุดารัตน์ บุญรอด (หญิง, อายุ 76 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G39" s="4" t="n">
@@ -4222,9 +4222,9 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>1. นางเสาวลักษณ์ พูนศิริ (หญิง, 25–44 ปี, พนักงานบริษัท)
-2. ด.ญ.วิไลลักษณ์ พูนศิริ (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-3. ด.ญ.วิลัยวรรณ พูนศิริ (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางเสาวลักษณ์ พูนศิริ (หญิง, อายุ 30 ปี, พนักงานบริษัท)
+2. ด.ญ.วิไลลักษณ์ พูนศิริ (หญิง, อายุ 10 ปี, นักเรียน/นักศึกษา)
+3. ด.ญ.วิลัยวรรณ พูนศิริ (หญิง, อายุ 8 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
@@ -4317,9 +4317,9 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>1. นางสุริยา กองประเสริฐ (หญิง, 60 ปีขึ้นไป, เกษตรกรรม)
-2. นายกรวิช กองประเสริฐ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-3. นางสาวเขมมิกา กองประเสริฐ (หญิง, 25–44 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
+          <t>1. นางสุริยา กองประเสริฐ (หญิง, อายุ 60 ปี, เกษตรกรรม)
+2. นายกรวิช กองประเสริฐ (ชาย, อายุ 62 ปี, เกษตรกรรม)
+3. นางสาวเขมมิกา กองประเสริฐ (หญิง, อายุ 25 ปี, รับราชการ/รัฐวิสาหกิจ)</t>
         </is>
       </c>
       <c r="G41" s="4" t="n">
@@ -4412,8 +4412,8 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>1. ทองสุข บุญธรรม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. บุญลือ บุญธรรม (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ทองสุข บุญธรรม (หญิง, อายุ 72 ปี, ไม่ได้ประกอบอาชีพ)
+2. บุญลือ บุญธรรม (ชาย, อายุ 75 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>1. ไพศล ทองพูน (ชาย, 45–59 ปี, รับจ้าง)</t>
+          <t>1. ไพศล ทองพูน (ชาย, อายุ 56 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G43" s="4" t="n">
@@ -4599,11 +4599,11 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>1. นางบังอ้อย พิษณุนาวิน (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นายจำเลียง บุญมี (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นางวันเพ็ญ ขันเงิน (หญิง, 25–44 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. ด.ช.ณัฐพัฒน์ สันเงิน (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-5. ด.ช.ภูมิพัฒน์ ขันเงิน (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นางบังอ้อย พิษณุนาวิน (หญิง, อายุ 63 ปี, ไม่ได้ประกอบอาชีพ)
+2. นายจำเลียง บุญมี (ชาย, อายุ 63 ปี, ไม่ได้ประกอบอาชีพ)
+3. นางวันเพ็ญ ขันเงิน (หญิง, อายุ 35 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. ด.ช.ณัฐพัฒน์ สันเงิน (ชาย, อายุ 12 ปี, นักเรียน/นักศึกษา)
+5. ด.ช.ภูมิพัฒน์ ขันเงิน (ชาย, อายุ 4 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>1. มานัด ทองพูน (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. มานัด ทองพูน (ชาย, อายุ 83 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G45" s="4" t="n">
@@ -4789,10 +4789,10 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>1. บุญเลิศ ทองคำ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. อนงค์ ทองคำ (หญิง, 60 ปีขึ้นไป, เกษตรกรรม)
-3. อนุสิทธิ์ ทองคำ (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)
-4. เต็มวุฒิ ทองคำ (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. บุญเลิศ ทองคำ (ชาย, อายุ 69 ปี, เกษตรกรรม)
+2. อนงค์ ทองคำ (หญิง, อายุ 60 ปี, เกษตรกรรม)
+3. อนุสิทธิ์ ทองคำ (ชาย, อายุ 19 ปี, นักเรียน/นักศึกษา)
+4. เต็มวุฒิ ทองคำ (ชาย, อายุ 17 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
@@ -4885,9 +4885,9 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>1. นางอำพร รุ่งสว่าง (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางจริญ จิราวัฒ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายชูเกียรติ สมรักษา (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. นางอำพร รุ่งสว่าง (หญิง, อายุ 64 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางจริญ จิราวัฒ (หญิง, อายุ 84 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายชูเกียรติ สมรักษา (ชาย, อายุ 26 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G47" s="4" t="n">
@@ -4980,8 +4980,8 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>1. ไพเราะ มนต์ขจรเดชา (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ปรีชา บุญธรรม (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ไพเราะ มนต์ขจรเดชา (หญิง, อายุ 67 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. ปรีชา บุญธรรม (ชาย, อายุ 59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
@@ -5074,10 +5074,10 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>1. ปราโมทย์ รื่นรวย (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. สมหมาย รื่นรวย (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. สมมาตร รื่นรวย (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-4. กิตติมา รื่นรวย (หญิง, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ปราโมทย์ รื่นรวย (ชาย, อายุ 71 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. สมหมาย รื่นรวย (หญิง, อายุ 69 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. สมมาตร รื่นรวย (ชาย, อายุ 42 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+4. กิตติมา รื่นรวย (หญิง, อายุ 28 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G49" s="4" t="n">
@@ -5170,8 +5170,8 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>1. พรจิตร ทองสนธิ (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ฉัตรชัย ประสงค์เงิน (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. พรจิตร ทองสนธิ (หญิง, อายุ 63 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. ฉัตรชัย ประสงค์เงิน (ชาย, อายุ 64 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
@@ -5264,9 +5264,9 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>1. ลินนา ตันพาณิชย์ (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. วัฒนา บุญมี (ชาย, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-3. วรพจน์ บุญมี (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
+          <t>1. ลินนา ตันพาณิชย์ (หญิง, อายุ 56 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. วัฒนา บุญมี (ชาย, อายุ 61 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. วรพจน์ บุญมี (ชาย, อายุ 30 ปี, ค้าขาย/ธุรกิจส่วนตัว)</t>
         </is>
       </c>
       <c r="G51" s="4" t="n">
@@ -5359,14 +5359,14 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>1. วันเพ็ญ บุญรอด (หญิง, 60 ปีขึ้นไป, ข้าราชการบำนาญ)
-2. บรรเจิด บุญรอด (ชาย, 60 ปีขึ้นไป, ข้าราชการบำนาญ)
-3. วงศกร บุญรอด (ชาย, 60 ปีขึ้นไป, พนักงานบริษัท)
-4. วีรากร บุญรอด (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. วันเพ็ญ บุญรอด (หญิง, อายุ 65 ปี, ข้าราชการบำนาญ)
+2. บรรเจิด บุญรอด (ชาย, อายุ 66 ปี, ข้าราชการบำนาญ)
+3. วงศกร บุญรอด (ชาย, อายุ 38 ปี, พนักงานบริษัท)
+4. วีรากร บุญรอด (ชาย, อายุ 12 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
@@ -5455,12 +5455,12 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>1. นายประจวบ ทองสนธิ (ชาย, 60 ปีขึ้นไป, รับจ้าง)
-2. นางพุทธชาติ ทองสนธิ (หญิง, 45–59 ปี, แม่บ้าน)
-3. นายทศพล ทองสนธิ (ชาย, 25–44 ปี, รับจ้าง)
-4. นายสกล ทองสนธิ (ชาย, 25–44 ปี, รับจ้าง)
-5. ด.ช.จักรกฤษณ์ ทองสนธิ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-6. ด.ช.ภพพิพัฒน์ ทองสนธิ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นายประจวบ ทองสนธิ (ชาย, อายุ 63 ปี, รับจ้าง)
+2. นางพุทธชาติ ทองสนธิ (หญิง, อายุ 59 ปี, แม่บ้าน)
+3. นายทศพล ทองสนธิ (ชาย, อายุ 33 ปี, รับจ้าง)
+4. นายสกล ทองสนธิ (ชาย, อายุ 30 ปี, รับจ้าง)
+5. ด.ช.จักรกฤษณ์ ทองสนธิ (ชาย, อายุ 14 ปี, นักเรียน/นักศึกษา)
+6. ด.ช.ภพพิพัฒน์ ทองสนธิ (ชาย, อายุ 8 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G53" s="4" t="n">
@@ -5553,8 +5553,8 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>1. ศิริญญา รื่นรวย (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. ณปภากร สุขพงศ์ไทย (หญิง, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. ศิริญญา รื่นรวย (หญิง, อายุ 45 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. ณปภากร สุขพงศ์ไทย (หญิง, อายุ 12 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
@@ -5647,11 +5647,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>1. นายมงคล พลอยสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางอรอุษา พลอยสมุทร (หญิง, 45–59 ปี, รับจ้าง)
-3. นางสาวนฤมล พลอยสมุทร (หญิง, 25–44 ปี, พนักงานบริษัท)
-4. นายอดิศร พลอยสมุทร (ชาย, 25–44 ปี, ช่างไฟฟ้า)
-5. ด.ญ.นฐพร พลอยสมุทร (หญิง, ต่ำกว่า 15 ปี, ยังไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายมงคล พลอยสมุทร (ชาย, อายุ 64 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางอรอุษา พลอยสมุทร (หญิง, อายุ 59 ปี, รับจ้าง)
+3. นางสาวนฤมล พลอยสมุทร (หญิง, อายุ 25 ปี, พนักงานบริษัท)
+4. นายอดิศร พลอยสมุทร (ชาย, อายุ 31 ปี, ช่างไฟฟ้า)
+5. ด.ญ.นฐพร พลอยสมุทร (หญิง, อายุ 1 ปี 10 เดือน, ยังไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G55" s="4" t="n">
@@ -5744,9 +5744,9 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>1. จำเนียร รัศมี (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. ปัญญารัตน์ รัศมี (หญิง, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-3. มาโนช นาคก่ำ (ชาย, 45–59 ปี, เกษตรกรรม)</t>
+          <t>1. จำเนียร รัศมี (หญิง, อายุ 71 ปี, ไม่ได้ประกอบอาชีพ)
+2. ปัญญารัตน์ รัศมี (หญิง, อายุ 50 ปี, รับราชการ/รัฐวิสาหกิจ)
+3. มาโนช นาคก่ำ (ชาย, อายุ 53 ปี, เกษตรกรรม)</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
@@ -5839,15 +5839,15 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>1. นางสาวดาราวรรณ ละมั่งทอง (หญิง, 60 ปีขึ้นไป, พนักงานบริษัท)
-2. นางสาวรัศมี เกตุแก้ว (หญิง, 15–24 ปี, พนักงานบริษัท)
-3. ด.ช.เตชินท์ ละมั่งทอง (ชาย, ต่ำกว่า 15 ปี, แรกเกิด)
-4. นายพีระวัฒน์ วงค์นิล (ชาย, 25–44 ปี, พนักงานบริษัท)
-5. นายธยธร เนียมชาติ (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสาวดาราวรรณ ละมั่งทอง (หญิง, อายุ 25 ปี, พนักงานบริษัท)
+2. นางสาวรัศมี เกตุแก้ว (หญิง, อายุ 22 ปี, พนักงานบริษัท)
+3. ด.ช.เตชินท์ ละมั่งทอง (ชาย, อายุ 2 เดือน, แรกเกิด)
+4. นายพีระวัฒน์ วงค์นิล (ชาย, อายุ 29 ปี, พนักงานบริษัท)
+5. นายธยธร เนียมชาติ (ชาย, อายุ 27 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
@@ -5936,8 +5936,8 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>1. สมร จันทร์ทร (หญิง, 60 ปีขึ้นไป, ค้าขาย/ธุรกิจส่วนตัว)
-2. ภิญญาธิดา มลขจรเดชา (หญิง, 15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. สมร จันทร์ทร (หญิง, อายุ 66 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. ภิญญาธิดา มลขจรเดชา (หญิง, อายุ 20 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
@@ -6030,7 +6030,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>1. มะลิวรรณ ชีวงษ์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. มะลิวรรณ ชีวงษ์ (หญิง, อายุ 72 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G59" s="4" t="n">
@@ -6123,8 +6123,8 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>1. สนธยา จันทร์ทร (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)
-2. ณัฐกร จันทร์ทร (ชาย, 15–24 ปี, รับจ้าง)</t>
+          <t>1. สนธยา จันทร์ทร (ชาย, อายุ 61 ปี, เกษตรกรรม)
+2. ณัฐกร จันทร์ทร (ชาย, อายุ 21 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
@@ -6217,9 +6217,9 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>1. ชวลิต รื่นเริง (ชาย, 45–59 ปี, รับจ้าง)
-2. ลัดดา ชีวงษ์ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. ภาคภูมิ รื่นเริง (ชาย, 45–59 ปี, รับจ้าง)</t>
+          <t>1. ชวลิต รื่นเริง (ชาย, อายุ 57 ปี, รับจ้าง)
+2. ลัดดา ชีวงษ์ (หญิง, อายุ 75 ปี, ไม่ได้ประกอบอาชีพ)
+3. ภาคภูมิ รื่นเริง (ชาย, อายุ 50 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G61" s="4" t="n">
@@ -6312,8 +6312,8 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>1. อนุชา เพชรชะรัด (ชาย, 45–59 ปี, รับจ้าง)
-2. ทองอยู่ เพชรชะรัด (ชาย, 60 ปีขึ้นไป, รับจ้าง)</t>
+          <t>1. อนุชา เพชรชะรัด (ชาย, อายุ 47 ปี, รับจ้าง)
+2. ทองอยู่ เพชรชะรัด (ชาย, อายุ 80 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
@@ -6406,9 +6406,9 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>1. นางบุญลือ จิตรวัฒน์ (หญิง, 60 ปีขึ้นไป, รับจ้าง)
-2. นายขวัญชัย ทองรัศมี (ชาย, 45–59 ปี, รับจ้าง)
-3. นายธีรศักศ์ ทองรัศมี (ชาย, 15–24 ปี, รับจ้าง)</t>
+          <t>1. นางบุญลือ จิตรวัฒน์ (หญิง, อายุ 72 ปี, รับจ้าง)
+2. นายขวัญชัย ทองรัศมี (ชาย, อายุ 50 ปี, รับจ้าง)
+3. นายธีรศักศ์ ทองรัศมี (ชาย, อายุ 23 ปี, รับจ้าง)</t>
         </is>
       </c>
       <c r="G63" s="4" t="n">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>1. นางอิ่ม ภักดีคำ (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางอิ่ม ภักดีคำ (หญิง, อายุ 84 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
@@ -6594,14 +6594,14 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>1. นางสมศรี แซ่ฮั่ง (หญิง, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-2. นายขจรศักดิ์ ฉั่วยู่เน้ย (ชาย, 25–44 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-3. นางสาวกุลธิชา พุทธม้าสี (หญิง, 25–44 ปี, รับราชการ/รัฐวิสาหกิจ)
-4. นายอนุชา ฉั่วยู่เน้ย (ชาย, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นางสมศรี แซ่ฮั่ง (หญิง, อายุ 63 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+2. นายขจรศักดิ์ ฉั่วยู่เน้ย (ชาย, อายุ 32 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+3. นางสาวกุลธิชา พุทธม้าสี (หญิง, อายุ 40 ปี, รับราชการ/รัฐวิสาหกิจ)
+4. นายอนุชา ฉั่วยู่เน้ย (ชาย, อายุ 38 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
@@ -6690,9 +6690,9 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>1. นายทศกร ทองชาวนา (ชาย, 45–59 ปี, รับจ้าง)
-2. นางสาวกมลพร พัคดีธรรม (หญิง, 45–59 ปี, พนักงานบริษัท)
-3. นายธีรการ ทองชาวนา (ชาย, 15–24 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. นายทศกร ทองชาวนา (ชาย, อายุ 51 ปี, รับจ้าง)
+2. นางสาวกมลพร พัคดีธรรม (หญิง, อายุ 52 ปี, พนักงานบริษัท)
+3. นายธีรการ ทองชาวนา (ชาย, อายุ 18 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
@@ -6785,10 +6785,10 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>1. สุจินดา เกาะประเสริฐ (ชาย, 45–59 ปี, รับราชการ/รัฐวิสาหกิจ)
-2. กรทิพย์ เกาะประเสริฐ (หญิง, 25–44 ปี, ผู้ช่วยผู้ใหญ่บ้าน)
-3. ชิษณุพงษ์ เกาะประเสริฐ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)
-4. ระพีพงษ์ เกาะประเสริฐ (ชาย, ต่ำกว่า 15 ปี, นักเรียน/นักศึกษา)</t>
+          <t>1. สุจินดา เกาะประเสริฐ (ชาย, อายุ 54 ปี, รับราชการ/รัฐวิสาหกิจ)
+2. กรทิพย์ เกาะประเสริฐ (หญิง, อายุ 48 ปี, ผู้ช่วยผู้ใหญ่บ้าน)
+3. ชิษณุพงษ์ เกาะประเสริฐ (ชาย, อายุ 13 ปี, นักเรียน/นักศึกษา)
+4. ระพีพงษ์ เกาะประเสริฐ (ชาย, อายุ 10 ปี, นักเรียน/นักศึกษา)</t>
         </is>
       </c>
       <c r="G67" s="4" t="n">
@@ -6881,7 +6881,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>1. ธงชัย โชคชัยฤทธิ์ (ชาย, 60 ปีขึ้นไป, เกษตรกรรม)</t>
+          <t>1. ธงชัย โชคชัยฤทธิ์ (ชาย, อายุ 60 ปี, เกษตรกรรม)</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
@@ -6974,12 +6974,12 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>1. นางพยอม เขียวสมุทร (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นายโสภา เขียวสมุทร (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายธีระยุทธ์ เขียวสมุทร (ชาย, 45–59 ปี, ค้าขาย/ธุรกิจส่วนตัว)
-4. นางกนกกร เขียวสมุทร (หญิง, 25–44 ปี, อสม)
-5. นายชวกร เขียวสมุทร (ชาย, 15–24 ปี, เรียนอยู่)
-6. นางสาวมณีรัตน์ เขียวสมุทร (หญิง, 25–44 ปี, เรียนอยู่)</t>
+          <t>1. นางพยอม เขียวสมุทร (หญิง, อายุ 85 ปี, ไม่ได้ประกอบอาชีพ)
+2. นายโสภา เขียวสมุทร (ชาย, อายุ 86 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายธีระยุทธ์ เขียวสมุทร (ชาย, อายุ 50 ปี, ค้าขาย/ธุรกิจส่วนตัว)
+4. นางกนกกร เขียวสมุทร (หญิง, อายุ 41 ปี, อสม)
+5. นายชวกร เขียวสมุทร (ชาย, อายุ 21 ปี, เรียนอยู่)
+6. นางสาวมณีรัตน์ เขียวสมุทร (หญิง, อายุ 18 ปี, เรียนอยู่)</t>
         </is>
       </c>
       <c r="G69" s="4" t="n">
@@ -7072,12 +7072,12 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>1. นายสันต์ รัศมี (ชาย, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-2. นางสำลี รัศมี (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)
-3. นายสุรชัย รัศมี (ชาย, 45–59 ปี, ไม่ได้ประกอบอาชีพ)
-4. นายอนพัฒน์ รัศมี (ชาย, 15–24 ปี, พนักงานบริษัท)
-5. นายสุพัฒน์ รัศมี (ชาย, 15–24 ปี, พนักงานบริษัท)
-6. นางสาววศิตา  เจ๊ะอาแส (หญิง, 25–44 ปี, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. นายสันต์ รัศมี (ชาย, อายุ 80 ปี, ไม่ได้ประกอบอาชีพ)
+2. นางสำลี รัศมี (หญิง, อายุ 75 ปี, ไม่ได้ประกอบอาชีพ)
+3. นายสุรชัย รัศมี (ชาย, อายุ 45 ปี, ไม่ได้ประกอบอาชีพ)
+4. นายอนพัฒน์ รัศมี (ชาย, อายุ 21 ปี, พนักงานบริษัท)
+5. นายสุพัฒน์ รัศมี (ชาย, อายุ 19 ปี, พนักงานบริษัท)
+6. นางสาววศิตา  เจ๊ะอาแส (หญิง, อายุ 26 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>1. ขวัญใจ ชื่นชม (หญิง, 60 ปีขึ้นไป, ไม่ได้ประกอบอาชีพ)</t>
+          <t>1. ขวัญใจ ชื่นชม (หญิง, อายุ 74 ปี, ไม่ได้ประกอบอาชีพ)</t>
         </is>
       </c>
       <c r="G71" s="4" t="n">
@@ -7423,10 +7423,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F2" s="6" t="n">
+        <v>56</v>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
@@ -7529,10 +7527,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F3" s="8" t="n">
+        <v>75</v>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
@@ -7643,10 +7639,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F4" s="6" t="n">
+        <v>87</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -7749,10 +7743,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F5" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
@@ -7863,10 +7855,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F6" s="6" t="n">
+        <v>17</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -7961,10 +7951,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F7" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
@@ -8079,10 +8067,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F8" s="6" t="n">
+        <v>52</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -8189,10 +8175,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F9" s="8" t="n">
+        <v>11</v>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
@@ -8299,10 +8283,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F10" s="6" t="n">
+        <v>66</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
@@ -8409,10 +8391,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F11" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
@@ -8523,10 +8503,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F12" s="6" t="n">
+        <v>35</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -8601,10 +8579,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F13" s="8" t="n">
+        <v>14</v>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -8679,10 +8655,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F14" s="6" t="n">
+        <v>56</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
@@ -8793,10 +8767,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F15" s="8" t="n">
+        <v>75</v>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
@@ -8903,10 +8875,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F16" s="6" t="n">
+        <v>74</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
@@ -9009,10 +8979,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F17" s="8" t="n">
+        <v>93</v>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
@@ -9127,10 +9095,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F18" s="6" t="n">
+        <v>87</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
@@ -9237,10 +9203,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F19" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
@@ -9343,10 +9307,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F20" s="6" t="n">
+        <v>59</v>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
@@ -9457,10 +9419,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F21" s="8" t="n">
+        <v>37</v>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
@@ -9563,10 +9523,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F22" s="6" t="n">
+        <v>33</v>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
@@ -9677,10 +9635,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F23" s="8" t="n">
+        <v>63</v>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
@@ -9783,10 +9739,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F24" s="6" t="n">
+        <v>30</v>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
@@ -9889,10 +9843,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F25" s="8" t="n">
+        <v>15</v>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
@@ -9995,10 +9947,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F26" s="6" t="n">
+        <v>69</v>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
@@ -10113,10 +10063,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F27" s="8" t="n">
+        <v>48</v>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
@@ -10223,10 +10171,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F28" s="6" t="n">
+        <v>18</v>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
@@ -10329,10 +10275,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F29" s="8" t="n">
+        <v>77</v>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
@@ -10447,10 +10391,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F30" s="6" t="n">
+        <v>73</v>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
@@ -10557,10 +10499,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F31" s="8" t="n">
+        <v>35</v>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
@@ -10667,10 +10607,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F32" s="6" t="n">
+        <v>79</v>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
@@ -10785,10 +10723,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F33" s="8" t="n">
+        <v>49</v>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
@@ -10899,10 +10835,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F34" s="6" t="n">
+        <v>73</v>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
@@ -11005,10 +10939,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F35" s="8" t="n">
+        <v>67</v>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
@@ -11119,10 +11051,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F36" s="6" t="n">
+        <v>47</v>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
@@ -11217,10 +11147,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F37" s="8" t="n">
+        <v>46</v>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
@@ -11315,10 +11243,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F38" s="6" t="n">
+        <v>45</v>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
@@ -11413,10 +11339,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F39" s="8" t="n">
+        <v>55</v>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
@@ -11531,10 +11455,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F40" s="6" t="n">
+        <v>58</v>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
@@ -11641,10 +11563,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F41" s="8" t="n">
+        <v>71</v>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
@@ -11759,10 +11679,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F42" s="6" t="n">
+        <v>78</v>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
@@ -11873,10 +11791,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F43" s="8" t="n">
+        <v>26</v>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
@@ -11979,10 +11895,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F44" s="6" t="n">
+        <v>40</v>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
@@ -12085,10 +11999,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F45" s="8" t="n">
+        <v>49</v>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
@@ -12203,10 +12115,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F46" s="6" t="n">
+        <v>49</v>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
@@ -12309,10 +12219,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F47" s="8" t="n">
+        <v>26</v>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
@@ -12415,10 +12323,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F48" s="6" t="n">
+        <v>24</v>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
@@ -12521,10 +12427,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F49" s="8" t="n">
+        <v>78</v>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
@@ -12639,10 +12543,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F50" s="6" t="n">
+        <v>84</v>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
@@ -12749,10 +12651,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F51" s="8" t="n">
+        <v>55</v>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
@@ -12859,10 +12759,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F52" s="6" t="n">
+        <v>57</v>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
@@ -12969,10 +12867,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F53" s="8" t="n">
+        <v>73</v>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
@@ -13083,10 +12979,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F54" s="6" t="n">
+        <v>71</v>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
@@ -13201,10 +13095,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F55" s="8" t="n">
+        <v>62</v>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
@@ -13319,10 +13211,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F56" s="6" t="n">
+        <v>34</v>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
@@ -13433,10 +13323,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F57" s="8" t="n">
+        <v>33</v>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
@@ -13539,10 +13427,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F58" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
@@ -13645,10 +13531,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F59" s="8" t="n">
+        <v>65</v>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
@@ -13751,10 +13635,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F60" s="6" t="n">
+        <v>29</v>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
@@ -13857,10 +13739,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F61" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F61" s="8" t="n">
+        <v>80</v>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
@@ -13975,10 +13855,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F62" s="6" t="n">
+        <v>80</v>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
@@ -14093,10 +13971,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F63" s="8" t="n">
+        <v>35</v>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
@@ -14171,10 +14047,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F64" s="6" t="n">
+        <v>61</v>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
@@ -14289,10 +14163,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F65" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F65" s="8" t="n">
+        <v>42</v>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
@@ -14399,10 +14271,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F66" s="6" t="n">
+        <v>11</v>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
@@ -14505,10 +14375,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F67" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F67" s="8" t="n">
+        <v>9</v>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
@@ -14611,10 +14479,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F68" s="6" t="n">
+        <v>45</v>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
@@ -14725,10 +14591,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F69" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F69" s="8" t="n">
+        <v>52</v>
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
@@ -14831,10 +14695,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F70" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
@@ -14933,10 +14795,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F71" s="8" t="n">
+        <v>71</v>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
@@ -15051,10 +14911,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F72" s="6" t="n">
+        <v>71</v>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
@@ -15165,10 +15023,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F73" s="8" t="n">
+        <v>69</v>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
@@ -15283,10 +15139,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F74" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F74" s="6" t="n">
+        <v>65</v>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
@@ -15393,10 +15247,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F75" s="8" t="n">
+        <v>89</v>
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
@@ -15511,10 +15363,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F76" s="6" t="n">
+        <v>77</v>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
@@ -15625,10 +15475,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F77" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F77" s="8" t="n">
+        <v>48</v>
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
@@ -15731,10 +15579,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F78" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F78" s="6" t="n">
+        <v>43</v>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
@@ -15837,10 +15683,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F79" s="8" t="n">
+        <v>17</v>
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
@@ -15943,10 +15787,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F80" s="6" t="n">
+        <v>17</v>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
@@ -16041,10 +15883,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F81" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F81" s="8" t="n">
+        <v>61</v>
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
@@ -16155,10 +15995,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F82" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F82" s="6" t="n">
+        <v>66</v>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
@@ -16265,10 +16103,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F83" s="8" t="n">
+        <v>23</v>
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
@@ -16343,10 +16179,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F84" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F84" s="6" t="n">
+        <v>23</v>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
@@ -16421,10 +16255,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F85" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F85" s="8" t="n">
+        <v>59</v>
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
@@ -16531,10 +16363,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F86" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F86" s="6" t="n">
+        <v>48</v>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
@@ -16641,10 +16471,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F87" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F87" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
@@ -16747,10 +16575,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F88" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F88" s="6" t="n">
+        <v>75</v>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
@@ -16861,10 +16687,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F89" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F89" s="8" t="n">
+        <v>75</v>
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
@@ -16971,10 +16795,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F90" s="6" t="n">
+        <v>65</v>
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
@@ -17085,10 +16907,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F91" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F91" s="8" t="n">
+        <v>83</v>
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
@@ -17203,10 +17023,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F92" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F92" s="6" t="n">
+        <v>42</v>
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
@@ -17317,10 +17135,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F93" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F93" s="8" t="n">
+        <v>64</v>
       </c>
       <c r="G93" s="9" t="inlineStr">
         <is>
@@ -17423,10 +17239,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F94" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F94" s="6" t="n">
+        <v>89</v>
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
@@ -17537,10 +17351,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F95" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F95" s="8" t="n">
+        <v>70</v>
       </c>
       <c r="G95" s="9" t="inlineStr">
         <is>
@@ -17647,10 +17459,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F96" s="6" t="n">
+        <v>65</v>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
@@ -17761,10 +17571,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F97" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F97" s="8" t="n">
+        <v>48</v>
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
@@ -17879,10 +17687,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F98" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F98" s="6" t="n">
+        <v>69</v>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
@@ -17997,10 +17803,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F99" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F99" s="8" t="n">
+        <v>21</v>
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
@@ -18103,10 +17907,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F100" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F100" s="6" t="n">
+        <v>22</v>
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
@@ -18209,10 +18011,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F101" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F101" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
@@ -18287,10 +18087,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F102" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F102" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
@@ -18365,10 +18163,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F103" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F103" s="8" t="n">
+        <v>68</v>
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
@@ -18475,10 +18271,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F104" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F104" s="6" t="n">
+        <v>48</v>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
@@ -18581,10 +18375,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F105" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F105" s="8" t="n">
+        <v>57</v>
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
@@ -18699,10 +18491,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F106" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F106" s="6" t="n">
+        <v>58</v>
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
@@ -18809,10 +18599,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F107" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F107" s="8" t="n">
+        <v>54</v>
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
@@ -18919,10 +18707,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F108" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F108" s="6" t="n">
+        <v>76</v>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
@@ -19037,10 +18823,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F109" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F109" s="8" t="n">
+        <v>30</v>
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
@@ -19151,10 +18935,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F110" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F110" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="G110" s="7" t="inlineStr">
         <is>
@@ -19253,10 +19035,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F111" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F111" s="8" t="n">
+        <v>8</v>
       </c>
       <c r="G111" s="9" t="inlineStr">
         <is>
@@ -19351,10 +19131,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F112" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F112" s="6" t="n">
+        <v>60</v>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
@@ -19465,10 +19243,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F113" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F113" s="8" t="n">
+        <v>62</v>
       </c>
       <c r="G113" s="9" t="inlineStr">
         <is>
@@ -19575,10 +19351,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F114" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F114" s="6" t="n">
+        <v>25</v>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
@@ -19689,10 +19463,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F115" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F115" s="8" t="n">
+        <v>72</v>
       </c>
       <c r="G115" s="9" t="inlineStr">
         <is>
@@ -19807,10 +19579,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F116" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F116" s="6" t="n">
+        <v>75</v>
       </c>
       <c r="G116" s="7" t="inlineStr">
         <is>
@@ -19917,10 +19687,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F117" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F117" s="8" t="n">
+        <v>56</v>
       </c>
       <c r="G117" s="9" t="inlineStr">
         <is>
@@ -20015,10 +19783,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F118" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F118" s="6" t="n">
+        <v>63</v>
       </c>
       <c r="G118" s="7" t="inlineStr">
         <is>
@@ -20133,10 +19899,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F119" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F119" s="8" t="n">
+        <v>63</v>
       </c>
       <c r="G119" s="9" t="inlineStr">
         <is>
@@ -20243,10 +20007,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F120" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F120" s="6" t="n">
+        <v>35</v>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
@@ -20357,10 +20119,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F121" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F121" s="8" t="n">
+        <v>12</v>
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
@@ -20463,10 +20223,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F122" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F122" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="G122" s="7" t="inlineStr">
         <is>
@@ -20569,10 +20327,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F123" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F123" s="8" t="n">
+        <v>83</v>
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
@@ -20675,10 +20431,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F124" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F124" s="6" t="n">
+        <v>69</v>
       </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
@@ -20785,10 +20539,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F125" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F125" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
@@ -20903,10 +20655,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F126" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F126" s="6" t="n">
+        <v>19</v>
       </c>
       <c r="G126" s="7" t="inlineStr">
         <is>
@@ -21009,10 +20759,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F127" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F127" s="8" t="n">
+        <v>17</v>
       </c>
       <c r="G127" s="9" t="inlineStr">
         <is>
@@ -21111,10 +20859,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F128" s="6" t="n">
+        <v>64</v>
       </c>
       <c r="G128" s="7" t="inlineStr">
         <is>
@@ -21225,10 +20971,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F129" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F129" s="8" t="n">
+        <v>84</v>
       </c>
       <c r="G129" s="9" t="inlineStr">
         <is>
@@ -21343,10 +21087,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F130" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F130" s="6" t="n">
+        <v>26</v>
       </c>
       <c r="G130" s="7" t="inlineStr">
         <is>
@@ -21461,10 +21203,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F131" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F131" s="8" t="n">
+        <v>67</v>
       </c>
       <c r="G131" s="9" t="inlineStr">
         <is>
@@ -21579,10 +21319,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F132" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F132" s="6" t="n">
+        <v>59</v>
       </c>
       <c r="G132" s="7" t="inlineStr">
         <is>
@@ -21689,10 +21427,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F133" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F133" s="8" t="n">
+        <v>71</v>
       </c>
       <c r="G133" s="9" t="inlineStr">
         <is>
@@ -21799,10 +21535,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F134" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F134" s="6" t="n">
+        <v>69</v>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
@@ -21917,10 +21651,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F135" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F135" s="8" t="n">
+        <v>42</v>
       </c>
       <c r="G135" s="9" t="inlineStr">
         <is>
@@ -22027,10 +21759,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F136" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F136" s="6" t="n">
+        <v>28</v>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
@@ -22141,10 +21871,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F137" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F137" s="8" t="n">
+        <v>63</v>
       </c>
       <c r="G137" s="9" t="inlineStr">
         <is>
@@ -22259,10 +21987,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F138" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F138" s="6" t="n">
+        <v>64</v>
       </c>
       <c r="G138" s="7" t="inlineStr">
         <is>
@@ -22369,10 +22095,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F139" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F139" s="8" t="n">
+        <v>56</v>
       </c>
       <c r="G139" s="9" t="inlineStr">
         <is>
@@ -22483,10 +22207,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F140" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F140" s="6" t="n">
+        <v>61</v>
       </c>
       <c r="G140" s="7" t="inlineStr">
         <is>
@@ -22589,10 +22311,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F141" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F141" s="8" t="n">
+        <v>30</v>
       </c>
       <c r="G141" s="9" t="inlineStr">
         <is>
@@ -22699,10 +22419,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F142" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F142" s="6" t="n">
+        <v>65</v>
       </c>
       <c r="G142" s="7" t="inlineStr">
         <is>
@@ -22817,10 +22535,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F143" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F143" s="8" t="n">
+        <v>66</v>
       </c>
       <c r="G143" s="9" t="inlineStr">
         <is>
@@ -22927,10 +22643,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F144" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F144" s="6" t="n">
+        <v>38</v>
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
@@ -23037,10 +22751,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F145" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F145" s="8" t="n">
+        <v>12</v>
       </c>
       <c r="G145" s="9" t="inlineStr">
         <is>
@@ -23147,10 +22859,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F146" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F146" s="6" t="n">
+        <v>63</v>
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
@@ -23253,10 +22963,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F147" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F147" s="8" t="n">
+        <v>59</v>
       </c>
       <c r="G147" s="9" t="inlineStr">
         <is>
@@ -23367,10 +23075,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F148" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F148" s="6" t="n">
+        <v>33</v>
       </c>
       <c r="G148" s="7" t="inlineStr">
         <is>
@@ -23473,10 +23179,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F149" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F149" s="8" t="n">
+        <v>30</v>
       </c>
       <c r="G149" s="9" t="inlineStr">
         <is>
@@ -23579,10 +23283,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F150" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F150" s="6" t="n">
+        <v>14</v>
       </c>
       <c r="G150" s="7" t="inlineStr">
         <is>
@@ -23689,10 +23391,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F151" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F151" s="8" t="n">
+        <v>8</v>
       </c>
       <c r="G151" s="9" t="inlineStr">
         <is>
@@ -23795,10 +23495,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F152" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F152" s="6" t="n">
+        <v>45</v>
       </c>
       <c r="G152" s="7" t="inlineStr">
         <is>
@@ -23909,10 +23607,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F153" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F153" s="8" t="n">
+        <v>12</v>
       </c>
       <c r="G153" s="9" t="inlineStr">
         <is>
@@ -24019,10 +23715,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F154" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F154" s="6" t="n">
+        <v>64</v>
       </c>
       <c r="G154" s="7" t="inlineStr">
         <is>
@@ -24125,10 +23819,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F155" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F155" s="8" t="n">
+        <v>59</v>
       </c>
       <c r="G155" s="9" t="inlineStr">
         <is>
@@ -24239,10 +23931,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F156" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F156" s="6" t="n">
+        <v>25</v>
       </c>
       <c r="G156" s="7" t="inlineStr">
         <is>
@@ -24353,10 +24043,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F157" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F157" s="8" t="n">
+        <v>31</v>
       </c>
       <c r="G157" s="9" t="inlineStr">
         <is>
@@ -24461,7 +24149,7 @@
       </c>
       <c r="F158" s="6" t="inlineStr">
         <is>
-          <t>ต่ำกว่า 15 ปี</t>
+          <t>1 ปี 10 เดือน</t>
         </is>
       </c>
       <c r="G158" s="7" t="inlineStr">
@@ -24561,10 +24249,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F159" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F159" s="8" t="n">
+        <v>71</v>
       </c>
       <c r="G159" s="9" t="inlineStr">
         <is>
@@ -24671,10 +24357,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F160" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F160" s="6" t="n">
+        <v>50</v>
       </c>
       <c r="G160" s="7" t="inlineStr">
         <is>
@@ -24781,10 +24465,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F161" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F161" s="8" t="n">
+        <v>53</v>
       </c>
       <c r="G161" s="9" t="inlineStr">
         <is>
@@ -24891,10 +24573,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F162" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F162" s="6" t="n">
+        <v>25</v>
       </c>
       <c r="G162" s="7" t="inlineStr">
         <is>
@@ -25005,10 +24685,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F163" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F163" s="8" t="n">
+        <v>22</v>
       </c>
       <c r="G163" s="9" t="inlineStr">
         <is>
@@ -25121,7 +24799,7 @@
       </c>
       <c r="F164" s="6" t="inlineStr">
         <is>
-          <t>ต่ำกว่า 15 ปี</t>
+          <t>2 เดือน</t>
         </is>
       </c>
       <c r="G164" s="7" t="inlineStr">
@@ -25225,10 +24903,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F165" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F165" s="8" t="n">
+        <v>29</v>
       </c>
       <c r="G165" s="9" t="inlineStr">
         <is>
@@ -25331,10 +25007,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F166" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F166" s="6" t="n">
+        <v>27</v>
       </c>
       <c r="G166" s="7" t="inlineStr">
         <is>
@@ -25437,10 +25111,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F167" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F167" s="8" t="n">
+        <v>66</v>
       </c>
       <c r="G167" s="9" t="inlineStr">
         <is>
@@ -25551,10 +25223,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F168" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F168" s="6" t="n">
+        <v>20</v>
       </c>
       <c r="G168" s="7" t="inlineStr">
         <is>
@@ -25637,10 +25307,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F169" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F169" s="8" t="n">
+        <v>72</v>
       </c>
       <c r="G169" s="9" t="inlineStr">
         <is>
@@ -25743,10 +25411,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F170" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F170" s="6" t="n">
+        <v>61</v>
       </c>
       <c r="G170" s="7" t="inlineStr">
         <is>
@@ -25853,10 +25519,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F171" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F171" s="8" t="n">
+        <v>21</v>
       </c>
       <c r="G171" s="9" t="inlineStr">
         <is>
@@ -25955,10 +25619,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F172" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F172" s="6" t="n">
+        <v>57</v>
       </c>
       <c r="G172" s="7" t="inlineStr">
         <is>
@@ -26061,10 +25723,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F173" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F173" s="8" t="n">
+        <v>75</v>
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
@@ -26167,10 +25827,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F174" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F174" s="6" t="n">
+        <v>50</v>
       </c>
       <c r="G174" s="7" t="inlineStr">
         <is>
@@ -26245,10 +25903,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F175" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F175" s="8" t="n">
+        <v>47</v>
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
@@ -26347,10 +26003,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F176" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F176" s="6" t="n">
+        <v>80</v>
       </c>
       <c r="G176" s="7" t="inlineStr">
         <is>
@@ -26453,10 +26107,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F177" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F177" s="8" t="n">
+        <v>72</v>
       </c>
       <c r="G177" s="9" t="inlineStr">
         <is>
@@ -26567,10 +26219,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F178" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F178" s="6" t="n">
+        <v>50</v>
       </c>
       <c r="G178" s="7" t="inlineStr">
         <is>
@@ -26673,10 +26323,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F179" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F179" s="8" t="n">
+        <v>23</v>
       </c>
       <c r="G179" s="9" t="inlineStr">
         <is>
@@ -26779,10 +26427,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F180" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F180" s="6" t="n">
+        <v>84</v>
       </c>
       <c r="G180" s="7" t="inlineStr">
         <is>
@@ -26889,10 +26535,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F181" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F181" s="8" t="n">
+        <v>63</v>
       </c>
       <c r="G181" s="9" t="inlineStr">
         <is>
@@ -27007,10 +26651,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F182" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F182" s="6" t="n">
+        <v>32</v>
       </c>
       <c r="G182" s="7" t="inlineStr">
         <is>
@@ -27113,10 +26755,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F183" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F183" s="8" t="n">
+        <v>40</v>
       </c>
       <c r="G183" s="9" t="inlineStr">
         <is>
@@ -27227,10 +26867,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F184" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F184" s="6" t="n">
+        <v>38</v>
       </c>
       <c r="G184" s="7" t="inlineStr">
         <is>
@@ -27329,10 +26967,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F185" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F185" s="8" t="n">
+        <v>51</v>
       </c>
       <c r="G185" s="9" t="inlineStr">
         <is>
@@ -27439,10 +27075,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F186" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F186" s="6" t="n">
+        <v>52</v>
       </c>
       <c r="G186" s="7" t="inlineStr">
         <is>
@@ -27557,10 +27191,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F187" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F187" s="8" t="n">
+        <v>18</v>
       </c>
       <c r="G187" s="9" t="inlineStr">
         <is>
@@ -27663,10 +27295,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F188" s="6" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F188" s="6" t="n">
+        <v>54</v>
       </c>
       <c r="G188" s="7" t="inlineStr">
         <is>
@@ -27765,10 +27395,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F189" s="8" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F189" s="8" t="n">
+        <v>48</v>
       </c>
       <c r="G189" s="9" t="inlineStr">
         <is>
@@ -27871,10 +27499,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F190" s="6" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F190" s="6" t="n">
+        <v>13</v>
       </c>
       <c r="G190" s="7" t="inlineStr">
         <is>
@@ -27965,10 +27591,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F191" s="8" t="inlineStr">
-        <is>
-          <t>ต่ำกว่า 15 ปี</t>
-        </is>
+      <c r="F191" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="G191" s="9" t="inlineStr">
         <is>
@@ -28059,10 +27683,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F192" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F192" s="6" t="n">
+        <v>60</v>
       </c>
       <c r="G192" s="7" t="inlineStr">
         <is>
@@ -28165,10 +27787,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F193" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F193" s="8" t="n">
+        <v>85</v>
       </c>
       <c r="G193" s="9" t="inlineStr">
         <is>
@@ -28283,10 +27903,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F194" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F194" s="6" t="n">
+        <v>86</v>
       </c>
       <c r="G194" s="7" t="inlineStr">
         <is>
@@ -28393,10 +28011,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F195" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F195" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="G195" s="9" t="inlineStr">
         <is>
@@ -28503,10 +28119,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F196" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F196" s="6" t="n">
+        <v>41</v>
       </c>
       <c r="G196" s="7" t="inlineStr">
         <is>
@@ -28621,10 +28235,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F197" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F197" s="8" t="n">
+        <v>21</v>
       </c>
       <c r="G197" s="9" t="inlineStr">
         <is>
@@ -28727,10 +28339,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F198" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F198" s="6" t="n">
+        <v>18</v>
       </c>
       <c r="G198" s="7" t="inlineStr">
         <is>
@@ -28841,10 +28451,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F199" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F199" s="8" t="n">
+        <v>80</v>
       </c>
       <c r="G199" s="9" t="inlineStr">
         <is>
@@ -28947,10 +28555,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F200" s="6" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F200" s="6" t="n">
+        <v>75</v>
       </c>
       <c r="G200" s="7" t="inlineStr">
         <is>
@@ -29065,10 +28671,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F201" s="8" t="inlineStr">
-        <is>
-          <t>45–59 ปี</t>
-        </is>
+      <c r="F201" s="8" t="n">
+        <v>45</v>
       </c>
       <c r="G201" s="9" t="inlineStr">
         <is>
@@ -29171,10 +28775,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F202" s="6" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F202" s="6" t="n">
+        <v>21</v>
       </c>
       <c r="G202" s="7" t="inlineStr">
         <is>
@@ -29277,10 +28879,8 @@
           <t>ชาย</t>
         </is>
       </c>
-      <c r="F203" s="8" t="inlineStr">
-        <is>
-          <t>15–24 ปี</t>
-        </is>
+      <c r="F203" s="8" t="n">
+        <v>19</v>
       </c>
       <c r="G203" s="9" t="inlineStr">
         <is>
@@ -29383,10 +28983,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F204" s="6" t="inlineStr">
-        <is>
-          <t>25–44 ปี</t>
-        </is>
+      <c r="F204" s="6" t="n">
+        <v>26</v>
       </c>
       <c r="G204" s="7" t="inlineStr">
         <is>
@@ -29497,10 +29095,8 @@
           <t>หญิง</t>
         </is>
       </c>
-      <c r="F205" s="8" t="inlineStr">
-        <is>
-          <t>60 ปีขึ้นไป</t>
-        </is>
+      <c r="F205" s="8" t="n">
+        <v>74</v>
       </c>
       <c r="G205" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Women's Health & Contraception sheet to Excel file
</commit_message>
<xml_diff>
--- a/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
+++ b/สรุปข้อมูลสุขภาพรายครอบครัว_ตำบลบางหัก_ม1.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ข้อมูลสรุปแยกรายบ้าน (70 หลัง)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ข้อมูลสมาชิกรายบุคคล (204 คน)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สุขภาพสตรีและการคุมกำเนิด" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +38,41 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Sarabun"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Sarabun"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Sarabun"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Sarabun"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Sarabun"/>
+      <b val="1"/>
+      <color rgb="009F1239"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Sarabun"/>
+      <b val="1"/>
+      <color rgb="00115E59"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,8 +91,26 @@
         <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F43F5E"/>
+        <bgColor rgb="00F43F5E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4E6"/>
+        <bgColor rgb="00FFE4E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCFBF1"/>
+        <bgColor rgb="00CCFBF1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -80,11 +132,25 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -112,6 +178,30 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -29180,4 +29270,2456 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H77"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="86" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="59" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>สรุปสถิติการตรวจคัดกรองมะเร็งสตรีและการคุมกำเนิด ตำบลบางหัก หมู่ 1 (Nหญิง = 97 คน)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>ตารางที่ 1: สรุป 3 ตัวชี้วัดสำคัญด้านสุขภาพสตรีและการวางแผนครอบครัว</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>ตัวชี้วัด / บริการสุขภาพ</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>กลุ่มเป้าหมาย</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>จำนวนเป้าหมาย (คน)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>ตรวจแล้ว / คุมกำเนิด (คน)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>ร้อยละ (%)</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>ยังไม่ตรวจ / ไม่คุม (คน)</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>ร้อยละ (%)</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>ผลการตรวจ / วิธีการเด่น</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>1. การตรวจคัดกรองมะเร็งปากมดลูก</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>สตรีอายุ 30–60 ปี</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>56.25%</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>43.75%</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>ผลปกติ 100% (Pap Smear / HPV DNA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>2. การตรวจคัดกรองมะเร็งเต้านม</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>สตรีอายุ 30–70 ปี</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>80.00%</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>20.00%</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>ผลปกติ 100% (คลำตรวจตนเอง / จนท.สาธารณสุข)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>3. การคุมกำเนิดในหญิงวัยเจริญพันธุ์ (รวมทั้งหมด)</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>หญิงอายุ 15–49 ปี</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>20.69%</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>13.79%</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>ยาฉีด 4 ราย (66.7%), ยาเม็ด 1, ยาเม็ด+ฝัง 1 (โสด 19 คน)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   * คิดเฉพาะกลุ่มที่ตอบคำถามการคุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>หญิงอายุ 15–49 ปี</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>60.00%</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>40.00%</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>กลุ่มไม่คุม 4 ราย มี 1 รายระบุว่าต้องการมีบุตร</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>ตารางที่ 2: รายชื่อสตรีกลุ่มเป้าหมายคัดกรองมะเร็งปากมดลูก (อายุ 30–60 ปี, N=32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>ลำดับ</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>บ้านเลขที่</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>ชื่อ-สกุล</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>อายุ (ปี)</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>การตรวจคัดกรอง</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>วิธีการตรวจ</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>ผลการตรวจ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวเพ็ญนภา บุญเสริม</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>จำไม่ได้</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>นางภิรมณ์พร บุญจันที</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>ไม่เคย</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>นฤมล บุญรอด</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>11/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>นางสุมาลี พวงโคสน</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวบุษรา เพชรรัตน์</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>6/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>นางนงนุช อยู่สุข</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ตรวจเพราะไม่ต้องการ</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>6/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>นางวรัญธร อยู่สุข</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ตรวจเพราะไม่ต้องการตรวจ</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวสุชิรา รื่นเริง</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>ไม่เคยตรวจเนื่องจากผู้รับบริการไม่มีครอบครัว</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>4/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>นางกมลรัตน์ คำประสิทธิ์</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>11/1</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>บุปผา ทิพย์กานนท์</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>4 ม.1</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>นางจุฑารัตน์ บุญคำ</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>เอมอร</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวธนพัฒน์ บุญช่วย</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวพรพิมล พูนศิริ</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวสาวินีย์ สีกาสี</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>ไม่เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>14/1</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>ปทุม เมฆจั่น</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>15/1</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>ภัทรทาดา ทองคำ</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>ไม่เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>20/2 หมู่1</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>ลภัสลดา ผู้ทัด</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>48/1</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>ธัญพร บุญรอด</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>ไมได้ไปหาหมอ</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G31" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>47/2</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>นางเสาวลักษณ์ พูนศิริ</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ต้องการตรวจ</t>
+        </is>
+      </c>
+      <c r="G32" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>3/2</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>นางสุริยา กองประเสริฐ</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F33" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G33" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>8/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>นางวันเพ็ญ ขันเงิน</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G34" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>อนงค์ ทองคำ</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G35" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>ลินนา ตันพาณิชย์</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G36" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="inlineStr">
+        <is>
+          <t>นางพุทธชาติ ทองสนธิ</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F37" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G37" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>14/5</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>ศิริญญา รื่นรวย</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G38" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>นางอรอุษา พลอยสมุทร</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>ไม่เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F39" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>ปัญญารัตน์ รัศมี</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>ไม่ระบุ</t>
+        </is>
+      </c>
+      <c r="F40" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>10/4</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวกุลธิชา พุทธม้าสี</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>ไม่เคยตรวจ เพราะไม่ต้องการตรวจ</t>
+        </is>
+      </c>
+      <c r="F41" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>40/4</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวกมลพร พัคดีธรรม</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F42" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G42" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>63/1 หมู่1</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>กรทิพย์ เกาะประเสริฐ</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F43" s="18" t="inlineStr">
+        <is>
+          <t>VIA</t>
+        </is>
+      </c>
+      <c r="G43" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="n">
+        <v>32</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>นางกนกกร เขียวสมุทร</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>เคยตรวจ</t>
+        </is>
+      </c>
+      <c r="F44" s="18" t="inlineStr">
+        <is>
+          <t>Pap Smear</t>
+        </is>
+      </c>
+      <c r="G44" s="18" t="inlineStr">
+        <is>
+          <t>ปกติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>ตารางที่ 3: รายชื่อหญิงวัยเจริญพันธุ์และการคุมกำเนิด (อายุ 15–49 ปี, N=29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>ลำดับ</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="inlineStr">
+        <is>
+          <t>บ้านเลขที่</t>
+        </is>
+      </c>
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>ชื่อ-สกุล</t>
+        </is>
+      </c>
+      <c r="D48" s="19" t="inlineStr">
+        <is>
+          <t>อายุ (ปี)</t>
+        </is>
+      </c>
+      <c r="E48" s="19" t="inlineStr">
+        <is>
+          <t>สถานะสมรส (ข้อ 42)</t>
+        </is>
+      </c>
+      <c r="F48" s="19" t="inlineStr">
+        <is>
+          <t>การคุมกำเนิด (ข้อ 43)</t>
+        </is>
+      </c>
+      <c r="G48" s="19" t="inlineStr">
+        <is>
+          <t>วิธีการคุมกำเนิด (ข้อ 44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวกัญญารัตน์ อัมไพ</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G49" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>6/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>นางวรัญธร อยู่สุข</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G50" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>25/2</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>เด็กหญิงธิติมา สาธุจรัญ</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G51" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวสุชิรา รื่นเริง</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G52" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>4/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>นางกมลรัตน์ คำประสิทธิ์</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F53" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G53" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>4 ม.1</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>นางจุฑารัตน์ บุญคำ</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>4 ม.1</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวอินทิรา ฉั่วยู่เน้ย</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F55" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G55" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวธนพัฒน์ บุญช่วย</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>คุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>ยาฉีดคุมกำเนิด</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวพรพิมล พูนศิริ</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวสาวินีย์ สีกาสี</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>คุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="inlineStr">
+        <is>
+          <t>ยาฉีดคุมกำเนิด</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>84/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>นางสาววัชนี พรหมพัฒน์</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G59" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>14/1</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>ปทุม เมฆจั่น</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>ไม่คุม</t>
+        </is>
+      </c>
+      <c r="G60" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>15/1</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>ภัทรทาดา ทองคำ</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G61" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>20/2 หมู่1</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>ลภัสลดา ผู้ทัด</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>20/2 หมู่1</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>รัตนาภร อเนก</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>47/2</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>นางเสาวลักษณ์ พูนศิริ</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>3/2</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวเขมมิกา กองประเสริฐ</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="inlineStr">
+        <is>
+          <t>ไม่คุม</t>
+        </is>
+      </c>
+      <c r="G65" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>8/1 ม.1</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>นางวันเพ็ญ ขันเงิน</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>คุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
+          <t>ยาเม็ดคุมกำเนิด</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>14/2</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>กิตติมา รื่นรวย</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>14/5</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>ศิริญญา รื่นรวย</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>คุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>ยาฉีดคุมกำเนิด</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวนฤมล พลอยสมุทร</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G69" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>49/4</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวดาราวรรณ ละมั่งทอง</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
+        <is>
+          <t>คุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="inlineStr">
+        <is>
+          <t>ยาฉีดคุมกำเนิด</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>49/4</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวรัศมี เกตุแก้ว</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>ไม่คุม</t>
+        </is>
+      </c>
+      <c r="G71" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>4/4 หมู่1</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>ภิญญาธิดา มลขจรเดชา</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>10/4</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวกุลธิชา พุทธม้าสี</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>ไม่คุมกำเนิดเพราะต้องการมีลูก</t>
+        </is>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>63/1 หมู่1</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>กรทิพย์ เกาะประเสริฐ</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F74" s="16" t="inlineStr">
+        <is>
+          <t>คุมกำเนิด</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>ยาเม็ดคุมกำเนิด, ยาฝังคุมกำเนิด</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>นางกนกกร เขียวสมุทร</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G75" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>นางสาวมณีรัตน์ เขียวสมุทร</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>ไม่มี</t>
+        </is>
+      </c>
+      <c r="F76" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G76" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>28/1</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>นางสาววศิตา  เจ๊ะอาแส</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>มี</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>ไม่ได้ระบุ</t>
+        </is>
+      </c>
+      <c r="G77" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>